<commit_message>
Expand state AI policy dataset
</commit_message>
<xml_diff>
--- a/india-ai-dashboard/data/dashboard.v1_industry_researched.xlsx
+++ b/india-ai-dashboard/data/dashboard.v1_industry_researched.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records" sheetId="1" r:id="R033c577705854785"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="Rbaf9e77f8b5c4623"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R521dcf35517e442f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Records" sheetId="1" r:id="R6070f87edac3489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" r:id="R9c736be42ea7420e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rfb8c67c593d94e62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,12 +29,22 @@
       <x:color rgb="FFFFFFFF"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -163,7 +173,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -195,6 +205,10 @@
     <x:xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -7315,445 +7329,3041 @@
       </x:c>
     </x:row>
     <x:row r="118">
-      <x:c r="A118"/>
-      <x:c r="B118"/>
-      <x:c r="C118"/>
-      <x:c r="D118"/>
-      <x:c r="E118"/>
-      <x:c r="F118"/>
-      <x:c r="G118"/>
-      <x:c r="H118"/>
-      <x:c r="I118"/>
-      <x:c r="J118"/>
-      <x:c r="K118"/>
-      <x:c r="L118"/>
-      <x:c r="M118"/>
-      <x:c r="N118"/>
-      <x:c r="O118"/>
-      <x:c r="P118"/>
-      <x:c r="Q118"/>
-      <x:c r="R118"/>
-      <x:c r="S118"/>
+      <x:c r="A118" t="str">
+        <x:v>ai-117</x:v>
+      </x:c>
+      <x:c r="B118" t="n">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>Government of Andhra Pradesh / Agriculture &amp; Allied Departments</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>AI-based pest and disease early-warning and satellite crop-risk analytics</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>Agriculture</x:v>
+      </x:c>
+      <x:c r="H118" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I118" t="str">
+        <x:v>Precision agriculture and crop-risk intelligence</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K118" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L118" t="str">
+        <x:v>AI predictive modelling, machine learning, satellite imagery, soil-moisture and weather analytics</x:v>
+      </x:c>
+      <x:c r="M118" t="str">
+        <x:v>An official agriculture white paper documents AI pest/disease alerts, crop classification and satellite-based risk analytics.</x:v>
+      </x:c>
+      <x:c r="N118" t="str">
+        <x:v>https://cse.ap.gov.in/DSE/gisInformation.do?filename=White+paper+Detailed+Notes+of+Agril+allied+dept.+23.12.pdf&amp;mode=viewStatisticstransfer</x:v>
+      </x:c>
+      <x:c r="O118" t="str"/>
+      <x:c r="P118" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q118" t="str"/>
+      <x:c r="R118" t="str"/>
+      <x:c r="S118" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
-      <x:c r="A119"/>
-      <x:c r="B119"/>
-      <x:c r="C119"/>
-      <x:c r="D119"/>
-      <x:c r="E119"/>
-      <x:c r="F119"/>
-      <x:c r="G119"/>
-      <x:c r="H119"/>
-      <x:c r="I119"/>
-      <x:c r="J119"/>
-      <x:c r="K119"/>
-      <x:c r="L119"/>
-      <x:c r="M119"/>
-      <x:c r="N119"/>
-      <x:c r="O119"/>
-      <x:c r="P119"/>
-      <x:c r="Q119"/>
-      <x:c r="R119"/>
-      <x:c r="S119"/>
+      <x:c r="A119" t="str">
+        <x:v>ai-118</x:v>
+      </x:c>
+      <x:c r="B119" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Tirupati</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>Sri Venkateswara University / APSCHE</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>Drones and Space Technologies Consortium with industry partners</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>Defence &amp; Aerospace</x:v>
+      </x:c>
+      <x:c r="H119" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I119" t="str">
+        <x:v>Drone and space technology research ecosystem</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K119" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L119" t="str">
+        <x:v>Unmanned systems, earth observation and space-technology collaboration</x:v>
+      </x:c>
+      <x:c r="M119" t="str">
+        <x:v>The official APPGCET/SVU page records the university's Drones and Space Technologies Consortium and participating industry partners.</x:v>
+      </x:c>
+      <x:c r="N119" t="str">
+        <x:v>https://cets.apsche.ap.gov.in/PGCET/PGCET_HomePages/AboutUs.aspx</x:v>
+      </x:c>
+      <x:c r="O119" t="str"/>
+      <x:c r="P119" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q119" t="str"/>
+      <x:c r="R119" t="str"/>
+      <x:c r="S119" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
-      <x:c r="A120"/>
-      <x:c r="B120"/>
-      <x:c r="C120"/>
-      <x:c r="D120"/>
-      <x:c r="E120"/>
-      <x:c r="F120"/>
-      <x:c r="G120"/>
-      <x:c r="H120"/>
-      <x:c r="I120"/>
-      <x:c r="J120"/>
-      <x:c r="K120"/>
-      <x:c r="L120"/>
-      <x:c r="M120"/>
-      <x:c r="N120"/>
-      <x:c r="O120"/>
-      <x:c r="P120"/>
-      <x:c r="Q120"/>
-      <x:c r="R120"/>
-      <x:c r="S120"/>
+      <x:c r="A120" t="str">
+        <x:v>ai-119</x:v>
+      </x:c>
+      <x:c r="B120" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>Andhra Pradesh Non-Resident Telugu Society</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>Advanced IT training covering artificial intelligence, data science and cloud</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>Education &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="H120" t="str">
+        <x:v>AI Talent &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="I120" t="str">
+        <x:v>AI and cloud workforce development</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>US$50 participant fee; not a programme investment commitment</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>Government training programme</x:v>
+      </x:c>
+      <x:c r="L120" t="str">
+        <x:v>Artificial intelligence, data science, Python, Hadoop, cybersecurity and AWS cloud</x:v>
+      </x:c>
+      <x:c r="M120" t="str">
+        <x:v>The official APNRTS portal lists AI and data-science training and an AWS cloud-practitioner programme.</x:v>
+      </x:c>
+      <x:c r="N120" t="str">
+        <x:v>https://apnrts.ap.gov.in/it_training</x:v>
+      </x:c>
+      <x:c r="O120" t="str"/>
+      <x:c r="P120" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q120" t="str"/>
+      <x:c r="R120" t="str"/>
+      <x:c r="S120" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
-      <x:c r="A121"/>
-      <x:c r="B121"/>
-      <x:c r="C121"/>
-      <x:c r="D121"/>
-      <x:c r="E121"/>
-      <x:c r="F121"/>
-      <x:c r="G121"/>
-      <x:c r="H121"/>
-      <x:c r="I121"/>
-      <x:c r="J121"/>
-      <x:c r="K121"/>
-      <x:c r="L121"/>
-      <x:c r="M121"/>
-      <x:c r="N121"/>
-      <x:c r="O121"/>
-      <x:c r="P121"/>
-      <x:c r="Q121"/>
-      <x:c r="R121"/>
-      <x:c r="S121"/>
+      <x:c r="A121" t="str">
+        <x:v>ai-120</x:v>
+      </x:c>
+      <x:c r="B121" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>ITE&amp;C Department, Government of Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>Government-data startup proofs of concept for citizen-centric administration</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H121" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I121" t="str">
+        <x:v>Government data and digital public-service delivery</x:v>
+      </x:c>
+      <x:c r="J121" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K121" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L121" t="str">
+        <x:v>AI, deep tech, drones and IoT applied to government problem statements</x:v>
+      </x:c>
+      <x:c r="M121" t="str">
+        <x:v>The official AP IT &amp; GCC Policy 4.0 describes startup POCs using government data and emerging technologies to improve public services.</x:v>
+      </x:c>
+      <x:c r="N121" t="str">
+        <x:v>https://apit.ap.gov.in/assets/files/AP%20IT%20%26%20GCC%20Policy%20%284%200%29%202024-2029_%20G%20O%20MS%20No.9%2C%20dt%2012%2012%202024.pdf</x:v>
+      </x:c>
+      <x:c r="O121" t="str"/>
+      <x:c r="P121" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q121" t="str"/>
+      <x:c r="R121" t="str"/>
+      <x:c r="S121" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
-      <x:c r="A122"/>
-      <x:c r="B122"/>
-      <x:c r="C122"/>
-      <x:c r="D122"/>
-      <x:c r="E122"/>
-      <x:c r="F122"/>
-      <x:c r="G122"/>
-      <x:c r="H122"/>
-      <x:c r="I122"/>
-      <x:c r="J122"/>
-      <x:c r="K122"/>
-      <x:c r="L122"/>
-      <x:c r="M122"/>
-      <x:c r="N122"/>
-      <x:c r="O122"/>
-      <x:c r="P122"/>
-      <x:c r="Q122"/>
-      <x:c r="R122"/>
-      <x:c r="S122"/>
+      <x:c r="A122" t="str">
+        <x:v>ai-121</x:v>
+      </x:c>
+      <x:c r="B122" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Tirupati</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>Sri Venkateswara University / SV Medical College</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>Interdisciplinary research collaboration addressing healthcare and science challenges</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>Healthcare</x:v>
+      </x:c>
+      <x:c r="H122" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I122" t="str">
+        <x:v>Health-science research and data-driven collaboration</x:v>
+      </x:c>
+      <x:c r="J122" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K122" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L122" t="str">
+        <x:v>Data science, machine learning and interdisciplinary healthcare research</x:v>
+      </x:c>
+      <x:c r="M122" t="str">
+        <x:v>The official APSCHE-hosted SVU profile documents AI/data-science programmes and collaboration with SV Medical College on healthcare research.</x:v>
+      </x:c>
+      <x:c r="N122" t="str">
+        <x:v>https://cets.apsche.ap.gov.in/PGCET/PGCET_HomePages/AboutUs.aspx</x:v>
+      </x:c>
+      <x:c r="O122" t="str"/>
+      <x:c r="P122" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q122" t="str"/>
+      <x:c r="R122" t="str"/>
+      <x:c r="S122" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
-      <x:c r="A123"/>
-      <x:c r="B123"/>
-      <x:c r="C123"/>
-      <x:c r="D123"/>
-      <x:c r="E123"/>
-      <x:c r="F123"/>
-      <x:c r="G123"/>
-      <x:c r="H123"/>
-      <x:c r="I123"/>
-      <x:c r="J123"/>
-      <x:c r="K123"/>
-      <x:c r="L123"/>
-      <x:c r="M123"/>
-      <x:c r="N123"/>
-      <x:c r="O123"/>
-      <x:c r="P123"/>
-      <x:c r="Q123"/>
-      <x:c r="R123"/>
-      <x:c r="S123"/>
+      <x:c r="A123" t="str">
+        <x:v>ai-122</x:v>
+      </x:c>
+      <x:c r="B123" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>Government of Andhra Pradesh / Industries &amp; Commerce Department</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>Industry 4.0 adoption framework under Electronics Manufacturing Policy 4.0</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H123" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="I123" t="str">
+        <x:v>AI-enabled smart manufacturing</x:v>
+      </x:c>
+      <x:c r="J123" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K123" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L123" t="str">
+        <x:v>AI, IoT, predictive operations and data-driven production optimization</x:v>
+      </x:c>
+      <x:c r="M123" t="str">
+        <x:v>The official electronics policy identifies AI and IoT as the two pillars of Industry 4.0 and commits to research and workforce support.</x:v>
+      </x:c>
+      <x:c r="N123" t="str">
+        <x:v>https://apmsmeone.ap.gov.in/MSMEONE/Data/ExistingPolicy/Andhra%20Pradesh%20Electronics%20Manufacturing%20policy%20%284.0%29%202024-29.pdf</x:v>
+      </x:c>
+      <x:c r="O123" t="str"/>
+      <x:c r="P123" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q123" t="str"/>
+      <x:c r="R123" t="str"/>
+      <x:c r="S123" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
-      <x:c r="A124"/>
-      <x:c r="B124"/>
-      <x:c r="C124"/>
-      <x:c r="D124"/>
-      <x:c r="E124"/>
-      <x:c r="F124"/>
-      <x:c r="G124"/>
-      <x:c r="H124"/>
-      <x:c r="I124"/>
-      <x:c r="J124"/>
-      <x:c r="K124"/>
-      <x:c r="L124"/>
-      <x:c r="M124"/>
-      <x:c r="N124"/>
-      <x:c r="O124"/>
-      <x:c r="P124"/>
-      <x:c r="Q124"/>
-      <x:c r="R124"/>
-      <x:c r="S124"/>
+      <x:c r="A124" t="str">
+        <x:v>ai-123</x:v>
+      </x:c>
+      <x:c r="B124" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>ITE&amp;C Department, Government of Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>Data Center Policy 4.0 targeting AI-capable advanced data centres</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="H124" t="str">
+        <x:v>Cloud &amp; Compute</x:v>
+      </x:c>
+      <x:c r="I124" t="str">
+        <x:v>AI-ready data-centre capacity and cloud infrastructure</x:v>
+      </x:c>
+      <x:c r="J124" t="str">
+        <x:v>Capacity target up to 1 GW; no row-specific investment amount disclosed</x:v>
+      </x:c>
+      <x:c r="K124" t="str">
+        <x:v>State policy target</x:v>
+      </x:c>
+      <x:c r="L124" t="str">
+        <x:v>Advanced data centres, multi-cloud workloads, AI vision analytics and natural-language processing</x:v>
+      </x:c>
+      <x:c r="M124" t="str">
+        <x:v>The official Data Center Policy 4.0 targets up to 1 GW of capacity and specifically seeks advanced data centres with AI capabilities.</x:v>
+      </x:c>
+      <x:c r="N124" t="str">
+        <x:v>https://apit.ap.gov.in/assets/files/Data%20Center%20Policy%20%284.0%29%202024-29.PDF</x:v>
+      </x:c>
+      <x:c r="O124" t="str"/>
+      <x:c r="P124" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q124" t="str"/>
+      <x:c r="R124" t="str"/>
+      <x:c r="S124" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
-      <x:c r="A125"/>
-      <x:c r="B125"/>
-      <x:c r="C125"/>
-      <x:c r="D125"/>
-      <x:c r="E125"/>
-      <x:c r="F125"/>
-      <x:c r="G125"/>
-      <x:c r="H125"/>
-      <x:c r="I125"/>
-      <x:c r="J125"/>
-      <x:c r="K125"/>
-      <x:c r="L125"/>
-      <x:c r="M125"/>
-      <x:c r="N125"/>
-      <x:c r="O125"/>
-      <x:c r="P125"/>
-      <x:c r="Q125"/>
-      <x:c r="R125"/>
-      <x:c r="S125"/>
+      <x:c r="A125" t="str">
+        <x:v>ai-124</x:v>
+      </x:c>
+      <x:c r="B125" t="n">
+        <x:v>2018</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>Real Time Governance Society, Government of Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>Real Time Governance analytics platform for responsive public administration</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H125" t="str">
+        <x:v>AI Strategy &amp; Governance</x:v>
+      </x:c>
+      <x:c r="I125" t="str">
+        <x:v>Real-time decision support and citizen-service governance</x:v>
+      </x:c>
+      <x:c r="J125" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K125" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L125" t="str">
+        <x:v>Machine learning, AI analytics, dashboards, sensors, drones and IoT</x:v>
+      </x:c>
+      <x:c r="M125" t="str">
+        <x:v>The official good-governance white paper describes RTGS use of machine-learning and AI tools for government analytics.</x:v>
+      </x:c>
+      <x:c r="N125" t="str">
+        <x:v>https://cse.ap.gov.in/DSE/gisInformation.do?filename=White+Paper+on+Good+Governance.pdf&amp;mode=viewStatisticstransfer</x:v>
+      </x:c>
+      <x:c r="O125" t="str"/>
+      <x:c r="P125" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q125" t="str"/>
+      <x:c r="R125" t="str"/>
+      <x:c r="S125" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="126">
-      <x:c r="A126"/>
-      <x:c r="B126"/>
-      <x:c r="C126"/>
-      <x:c r="D126"/>
-      <x:c r="E126"/>
-      <x:c r="F126"/>
-      <x:c r="G126"/>
-      <x:c r="H126"/>
-      <x:c r="I126"/>
-      <x:c r="J126"/>
-      <x:c r="K126"/>
-      <x:c r="L126"/>
-      <x:c r="M126"/>
-      <x:c r="N126"/>
-      <x:c r="O126"/>
-      <x:c r="P126"/>
-      <x:c r="Q126"/>
-      <x:c r="R126"/>
-      <x:c r="S126"/>
+      <x:c r="A126" t="str">
+        <x:v>ai-125</x:v>
+      </x:c>
+      <x:c r="B126" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>Government of Andhra Pradesh / Industries &amp; Commerce Department</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>Electronics Manufacturing Policy support for AI, IoT and advanced electronics</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H126" t="str">
+        <x:v>Semiconductor &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="I126" t="str">
+        <x:v>Electronics, smart hardware and responsible AI manufacturing</x:v>
+      </x:c>
+      <x:c r="J126" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K126" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L126" t="str">
+        <x:v>Electronics systems, AI, IoT and Industry 4.0</x:v>
+      </x:c>
+      <x:c r="M126" t="str">
+        <x:v>The official Electronics Manufacturing Policy 4.0 supports advanced electronics and an AI/IoT-enabled manufacturing ecosystem.</x:v>
+      </x:c>
+      <x:c r="N126" t="str">
+        <x:v>https://apmsmeone.ap.gov.in/MSMEONE/Data/ExistingPolicy/Andhra%20Pradesh%20Electronics%20Manufacturing%20policy%20%284.0%29%202024-29.pdf</x:v>
+      </x:c>
+      <x:c r="O126" t="str"/>
+      <x:c r="P126" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q126" t="str"/>
+      <x:c r="R126" t="str"/>
+      <x:c r="S126" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
-      <x:c r="A127"/>
-      <x:c r="B127"/>
-      <x:c r="C127"/>
-      <x:c r="D127"/>
-      <x:c r="E127"/>
-      <x:c r="F127"/>
-      <x:c r="G127"/>
-      <x:c r="H127"/>
-      <x:c r="I127"/>
-      <x:c r="J127"/>
-      <x:c r="K127"/>
-      <x:c r="L127"/>
-      <x:c r="M127"/>
-      <x:c r="N127"/>
-      <x:c r="O127"/>
-      <x:c r="P127"/>
-      <x:c r="Q127"/>
-      <x:c r="R127"/>
-      <x:c r="S127"/>
+      <x:c r="A127" t="str">
+        <x:v>ai-126</x:v>
+      </x:c>
+      <x:c r="B127" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>Andhra Pradesh</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>ITE&amp;C Department / Andhra Pradesh Innovation Society</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>Andhra Pradesh Innovation &amp; Startup Policy 4.0 (2024-29)</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H127" t="str">
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+      </x:c>
+      <x:c r="I127" t="str">
+        <x:v>Deep-tech, AI and ML startup incubation and incentives</x:v>
+      </x:c>
+      <x:c r="J127" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K127" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L127" t="str">
+        <x:v>AI, machine learning, deep tech and shared innovation infrastructure</x:v>
+      </x:c>
+      <x:c r="M127" t="str">
+        <x:v>The official government order approves the statewide Innovation &amp; Startup Policy 4.0 and its fiscal and non-fiscal support framework.</x:v>
+      </x:c>
+      <x:c r="N127" t="str">
+        <x:v>https://apit.ap.gov.in/assets/files/2025ITC_36058_MS3_E-2.pdf</x:v>
+      </x:c>
+      <x:c r="O127" t="str"/>
+      <x:c r="P127" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q127" t="str"/>
+      <x:c r="R127" t="str"/>
+      <x:c r="S127" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="128">
-      <x:c r="A128"/>
-      <x:c r="B128"/>
-      <x:c r="C128"/>
-      <x:c r="D128"/>
-      <x:c r="E128"/>
-      <x:c r="F128"/>
-      <x:c r="G128"/>
-      <x:c r="H128"/>
-      <x:c r="I128"/>
-      <x:c r="J128"/>
-      <x:c r="K128"/>
-      <x:c r="L128"/>
-      <x:c r="M128"/>
-      <x:c r="N128"/>
-      <x:c r="O128"/>
-      <x:c r="P128"/>
-      <x:c r="Q128"/>
-      <x:c r="R128"/>
-      <x:c r="S128"/>
+      <x:c r="A128" t="str">
+        <x:v>ai-127</x:v>
+      </x:c>
+      <x:c r="B128" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>Government of Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>Uttar Pradesh AI Mission (UP-AIM)</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H128" t="str">
+        <x:v>AI Strategy &amp; Governance</x:v>
+      </x:c>
+      <x:c r="I128" t="str">
+        <x:v>Statewide AI adoption across governance, economy and society</x:v>
+      </x:c>
+      <x:c r="J128" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K128" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L128" t="str">
+        <x:v>Responsible AI, sector use cases, foundational models and governance framework</x:v>
+      </x:c>
+      <x:c r="M128" t="str">
+        <x:v>The official 2026-27 budget highlights define UP-AIM and its eight implementation pillars.</x:v>
+      </x:c>
+      <x:c r="N128" t="str">
+        <x:v>https://information.up.gov.in/admin/UploadDocument/OtherPress/compressed_20022026041527Budget%20Highlights%20English.pdf</x:v>
+      </x:c>
+      <x:c r="O128" t="str"/>
+      <x:c r="P128" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q128" t="str"/>
+      <x:c r="R128" t="str"/>
+      <x:c r="S128" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="129">
-      <x:c r="A129"/>
-      <x:c r="B129"/>
-      <x:c r="C129"/>
-      <x:c r="D129"/>
-      <x:c r="E129"/>
-      <x:c r="F129"/>
-      <x:c r="G129"/>
-      <x:c r="H129"/>
-      <x:c r="I129"/>
-      <x:c r="J129"/>
-      <x:c r="K129"/>
-      <x:c r="L129"/>
-      <x:c r="M129"/>
-      <x:c r="N129"/>
-      <x:c r="O129"/>
-      <x:c r="P129"/>
-      <x:c r="Q129"/>
-      <x:c r="R129"/>
-      <x:c r="S129"/>
+      <x:c r="A129" t="str">
+        <x:v>ai-128</x:v>
+      </x:c>
+      <x:c r="B129" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>Government of Uttar Pradesh / Invest UP</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>UP AI Mission support for medical and pharmaceutical AI</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>Healthcare</x:v>
+      </x:c>
+      <x:c r="H129" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I129" t="str">
+        <x:v>AI integration in healthcare, medical technology and pharmaceuticals</x:v>
+      </x:c>
+      <x:c r="J129" t="str">
+        <x:v>₹2,000 crore over three years</x:v>
+      </x:c>
+      <x:c r="K129" t="str">
+        <x:v>State mission allocation</x:v>
+      </x:c>
+      <x:c r="L129" t="str">
+        <x:v>AI-enabled medical and pharmaceutical research, diagnostics and applications</x:v>
+      </x:c>
+      <x:c r="M129" t="str">
+        <x:v>Invest UP reports a ₹2,000 crore, three-year UP AI Mission allocation targeting AI integration in medical and pharmaceutical sectors.</x:v>
+      </x:c>
+      <x:c r="N129" t="str">
+        <x:v>https://invest.up.gov.in/uttar-pradesh-indias/</x:v>
+      </x:c>
+      <x:c r="O129" t="str">
+        <x:v>INR</x:v>
+      </x:c>
+      <x:c r="P129" s="2" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q129" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="R129" t="str"/>
+      <x:c r="S129" t="str">
+        <x:v>Parsed INR crore amount from the cited government source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
-      <x:c r="A130"/>
-      <x:c r="B130"/>
-      <x:c r="C130"/>
-      <x:c r="D130"/>
-      <x:c r="E130"/>
-      <x:c r="F130"/>
-      <x:c r="G130"/>
-      <x:c r="H130"/>
-      <x:c r="I130"/>
-      <x:c r="J130"/>
-      <x:c r="K130"/>
-      <x:c r="L130"/>
-      <x:c r="M130"/>
-      <x:c r="N130"/>
-      <x:c r="O130"/>
-      <x:c r="P130"/>
-      <x:c r="Q130"/>
-      <x:c r="R130"/>
-      <x:c r="S130"/>
+      <x:c r="A130" t="str">
+        <x:v>ai-129</x:v>
+      </x:c>
+      <x:c r="B130" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>Government of Uttar Pradesh / School Education</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>AI-ML curriculum and technology labs in government schools</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>Education &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="H130" t="str">
+        <x:v>AI Talent &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="I130" t="str">
+        <x:v>School-level AI literacy and technical skills</x:v>
+      </x:c>
+      <x:c r="J130" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K130" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L130" t="str">
+        <x:v>AI/ML curriculum and school technology laboratories</x:v>
+      </x:c>
+      <x:c r="M130" t="str">
+        <x:v>The official 2026-27 budget highlights report AI-ML curriculum in 150 schools and technology labs across government schools.</x:v>
+      </x:c>
+      <x:c r="N130" t="str">
+        <x:v>https://information.up.gov.in/admin/UploadDocument/OtherPress/compressed_20022026041527Budget%20Highlights%20English.pdf</x:v>
+      </x:c>
+      <x:c r="O130" t="str"/>
+      <x:c r="P130" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q130" t="str"/>
+      <x:c r="R130" t="str"/>
+      <x:c r="S130" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="131">
-      <x:c r="A131"/>
-      <x:c r="B131"/>
-      <x:c r="C131"/>
-      <x:c r="D131"/>
-      <x:c r="E131"/>
-      <x:c r="F131"/>
-      <x:c r="G131"/>
-      <x:c r="H131"/>
-      <x:c r="I131"/>
-      <x:c r="J131"/>
-      <x:c r="K131"/>
-      <x:c r="L131"/>
-      <x:c r="M131"/>
-      <x:c r="N131"/>
-      <x:c r="O131"/>
-      <x:c r="P131"/>
-      <x:c r="Q131"/>
-      <x:c r="R131"/>
-      <x:c r="S131"/>
+      <x:c r="A131" t="str">
+        <x:v>ai-130</x:v>
+      </x:c>
+      <x:c r="B131" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>Invest UP / Government of Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="F131" t="str">
+        <x:v>Uttar Pradesh Global Capability Centers Policy 2024</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="H131" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="I131" t="str">
+        <x:v>Enterprise technology, finance operations and advanced GCC services</x:v>
+      </x:c>
+      <x:c r="J131" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K131" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L131" t="str">
+        <x:v>Digital functions, R&amp;D, finance and back-office automation supported by cloud services</x:v>
+      </x:c>
+      <x:c r="M131" t="str">
+        <x:v>The official UP GCC policy defines advanced centres spanning IT, R&amp;D, finance and digital operations, with cloud-cost support.</x:v>
+      </x:c>
+      <x:c r="N131" t="str">
+        <x:v>https://invest.up.gov.in/up-gcc-policy-2024/</x:v>
+      </x:c>
+      <x:c r="O131" t="str"/>
+      <x:c r="P131" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q131" t="str"/>
+      <x:c r="R131" t="str"/>
+      <x:c r="S131" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
-      <x:c r="A132"/>
-      <x:c r="B132"/>
-      <x:c r="C132"/>
-      <x:c r="D132"/>
-      <x:c r="E132"/>
-      <x:c r="F132"/>
-      <x:c r="G132"/>
-      <x:c r="H132"/>
-      <x:c r="I132"/>
-      <x:c r="J132"/>
-      <x:c r="K132"/>
-      <x:c r="L132"/>
-      <x:c r="M132"/>
-      <x:c r="N132"/>
-      <x:c r="O132"/>
-      <x:c r="P132"/>
-      <x:c r="Q132"/>
-      <x:c r="R132"/>
-      <x:c r="S132"/>
+      <x:c r="A132" t="str">
+        <x:v>ai-131</x:v>
+      </x:c>
+      <x:c r="B132" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>U.P. Electronics Corporation Limited</x:v>
+      </x:c>
+      <x:c r="F132" t="str">
+        <x:v>Uttar Pradesh Data Center Policy implementation and project pipeline</x:v>
+      </x:c>
+      <x:c r="G132" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="H132" t="str">
+        <x:v>Cloud &amp; Compute</x:v>
+      </x:c>
+      <x:c r="I132" t="str">
+        <x:v>Hyperscale data-centre parks and compute infrastructure</x:v>
+      </x:c>
+      <x:c r="J132" t="str">
+        <x:v>₹21,342.90 crore proposed investment as of June 2025</x:v>
+      </x:c>
+      <x:c r="K132" t="str">
+        <x:v>Proposed investment tracked by state agency</x:v>
+      </x:c>
+      <x:c r="L132" t="str">
+        <x:v>Hyperscale data centres, edge data centres, cloud and mission-critical digital infrastructure</x:v>
+      </x:c>
+      <x:c r="M132" t="str">
+        <x:v>The official UPLC dashboard reports ₹21,342.90 crore of proposed data-centre investment and 644 MW capacity as of June 2025.</x:v>
+      </x:c>
+      <x:c r="N132" t="str">
+        <x:v>https://uplc.up.gov.in/en/page/uttar-pradesh-data-center-policy</x:v>
+      </x:c>
+      <x:c r="O132" t="str">
+        <x:v>INR</x:v>
+      </x:c>
+      <x:c r="P132" s="2" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q132" t="n">
+        <x:v>21342.9</x:v>
+      </x:c>
+      <x:c r="R132" t="str"/>
+      <x:c r="S132" t="str">
+        <x:v>Parsed INR crore amount from the cited government source.</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
-      <x:c r="A133"/>
-      <x:c r="B133"/>
-      <x:c r="C133"/>
-      <x:c r="D133"/>
-      <x:c r="E133"/>
-      <x:c r="F133"/>
-      <x:c r="G133"/>
-      <x:c r="H133"/>
-      <x:c r="I133"/>
-      <x:c r="J133"/>
-      <x:c r="K133"/>
-      <x:c r="L133"/>
-      <x:c r="M133"/>
-      <x:c r="N133"/>
-      <x:c r="O133"/>
-      <x:c r="P133"/>
-      <x:c r="Q133"/>
-      <x:c r="R133"/>
-      <x:c r="S133"/>
+      <x:c r="A133" t="str">
+        <x:v>ai-132</x:v>
+      </x:c>
+      <x:c r="B133" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>Government of Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>UP-AIM open data and datasets platform pillar</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H133" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I133" t="str">
+        <x:v>Open government data and AI-ready datasets</x:v>
+      </x:c>
+      <x:c r="J133" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K133" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L133" t="str">
+        <x:v>Open data, interoperable datasets and public-sector AI infrastructure</x:v>
+      </x:c>
+      <x:c r="M133" t="str">
+        <x:v>The official UP budget identifies an Open Data &amp; Datasets Platform as a core UP-AIM pillar.</x:v>
+      </x:c>
+      <x:c r="N133" t="str">
+        <x:v>https://information.up.gov.in/admin/UploadDocument/OtherPress/compressed_20022026041527Budget%20Highlights%20English.pdf</x:v>
+      </x:c>
+      <x:c r="O133" t="str"/>
+      <x:c r="P133" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q133" t="str"/>
+      <x:c r="R133" t="str"/>
+      <x:c r="S133" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
-      <x:c r="A134"/>
-      <x:c r="B134"/>
-      <x:c r="C134"/>
-      <x:c r="D134"/>
-      <x:c r="E134"/>
-      <x:c r="F134"/>
-      <x:c r="G134"/>
-      <x:c r="H134"/>
-      <x:c r="I134"/>
-      <x:c r="J134"/>
-      <x:c r="K134"/>
-      <x:c r="L134"/>
-      <x:c r="M134"/>
-      <x:c r="N134"/>
-      <x:c r="O134"/>
-      <x:c r="P134"/>
-      <x:c r="Q134"/>
-      <x:c r="R134"/>
-      <x:c r="S134"/>
+      <x:c r="A134" t="str">
+        <x:v>ai-133</x:v>
+      </x:c>
+      <x:c r="B134" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>Government of Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="F134" t="str">
+        <x:v>UP-AIM foundational-model adoption pillar</x:v>
+      </x:c>
+      <x:c r="G134" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H134" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I134" t="str">
+        <x:v>Foundational models and new AI technologies</x:v>
+      </x:c>
+      <x:c r="J134" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K134" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L134" t="str">
+        <x:v>Foundation models and cross-sector AI adoption</x:v>
+      </x:c>
+      <x:c r="M134" t="str">
+        <x:v>The official UP budget lists leveraging foundational models as one of UP-AIM's core pillars.</x:v>
+      </x:c>
+      <x:c r="N134" t="str">
+        <x:v>https://information.up.gov.in/admin/UploadDocument/OtherPress/compressed_20022026041527Budget%20Highlights%20English.pdf</x:v>
+      </x:c>
+      <x:c r="O134" t="str"/>
+      <x:c r="P134" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q134" t="str"/>
+      <x:c r="R134" t="str"/>
+      <x:c r="S134" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="135">
-      <x:c r="A135"/>
-      <x:c r="B135"/>
-      <x:c r="C135"/>
-      <x:c r="D135"/>
-      <x:c r="E135"/>
-      <x:c r="F135"/>
-      <x:c r="G135"/>
-      <x:c r="H135"/>
-      <x:c r="I135"/>
-      <x:c r="J135"/>
-      <x:c r="K135"/>
-      <x:c r="L135"/>
-      <x:c r="M135"/>
-      <x:c r="N135"/>
-      <x:c r="O135"/>
-      <x:c r="P135"/>
-      <x:c r="Q135"/>
-      <x:c r="R135"/>
-      <x:c r="S135"/>
+      <x:c r="A135" t="str">
+        <x:v>ai-134</x:v>
+      </x:c>
+      <x:c r="B135" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>Invest UP / UP Defence Industrial Corridor</x:v>
+      </x:c>
+      <x:c r="F135" t="str">
+        <x:v>Defence testing facilities and Centres of Excellence at IIT Kanpur and IIT-BHU</x:v>
+      </x:c>
+      <x:c r="G135" t="str">
+        <x:v>Defence &amp; Aerospace</x:v>
+      </x:c>
+      <x:c r="H135" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I135" t="str">
+        <x:v>Defence R&amp;D, UAV testing and advanced diagnostics</x:v>
+      </x:c>
+      <x:c r="J135" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K135" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L135" t="str">
+        <x:v>UAS testing, communications testing, materials research and AI/ML diagnostic solutions</x:v>
+      </x:c>
+      <x:c r="M135" t="str">
+        <x:v>The official Invest UP sector page documents defence testing facilities, funded CoEs and AI/ML diagnostic-solution opportunities.</x:v>
+      </x:c>
+      <x:c r="N135" t="str">
+        <x:v>https://invest.up.gov.in/defence-aerospace-sector/</x:v>
+      </x:c>
+      <x:c r="O135" t="str"/>
+      <x:c r="P135" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q135" t="str"/>
+      <x:c r="R135" t="str"/>
+      <x:c r="S135" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="136">
-      <x:c r="A136"/>
-      <x:c r="B136"/>
-      <x:c r="C136"/>
-      <x:c r="D136"/>
-      <x:c r="E136"/>
-      <x:c r="F136"/>
-      <x:c r="G136"/>
-      <x:c r="H136"/>
-      <x:c r="I136"/>
-      <x:c r="J136"/>
-      <x:c r="K136"/>
-      <x:c r="L136"/>
-      <x:c r="M136"/>
-      <x:c r="N136"/>
-      <x:c r="O136"/>
-      <x:c r="P136"/>
-      <x:c r="Q136"/>
-      <x:c r="R136"/>
-      <x:c r="S136"/>
+      <x:c r="A136" t="str">
+        <x:v>ai-135</x:v>
+      </x:c>
+      <x:c r="B136" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>Invest UP / Government of Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="F136" t="str">
+        <x:v>Uttar Pradesh Semiconductor Policy 2024</x:v>
+      </x:c>
+      <x:c r="G136" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H136" t="str">
+        <x:v>Semiconductor &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="I136" t="str">
+        <x:v>Semiconductor fabs, ATMP/OSAT, sensors and chip design</x:v>
+      </x:c>
+      <x:c r="J136" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K136" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L136" t="str">
+        <x:v>Semiconductor manufacturing, silicon photonics, sensor fabs and design-led R&amp;D</x:v>
+      </x:c>
+      <x:c r="M136" t="str">
+        <x:v>The official Invest UP semiconductor page documents the 2024 policy, eligible technologies and state R&amp;D/CoE support.</x:v>
+      </x:c>
+      <x:c r="N136" t="str">
+        <x:v>https://invest.up.gov.in/semiconductor-sector/</x:v>
+      </x:c>
+      <x:c r="O136" t="str"/>
+      <x:c r="P136" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q136" t="str"/>
+      <x:c r="R136" t="str"/>
+      <x:c r="S136" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="137">
-      <x:c r="A137"/>
-      <x:c r="B137"/>
-      <x:c r="C137"/>
-      <x:c r="D137"/>
-      <x:c r="E137"/>
-      <x:c r="F137"/>
-      <x:c r="G137"/>
-      <x:c r="H137"/>
-      <x:c r="I137"/>
-      <x:c r="J137"/>
-      <x:c r="K137"/>
-      <x:c r="L137"/>
-      <x:c r="M137"/>
-      <x:c r="N137"/>
-      <x:c r="O137"/>
-      <x:c r="P137"/>
-      <x:c r="Q137"/>
-      <x:c r="R137"/>
-      <x:c r="S137"/>
+      <x:c r="A137" t="str">
+        <x:v>ai-136</x:v>
+      </x:c>
+      <x:c r="B137" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Uttar Pradesh</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>StartinUP / Department of IT &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="F137" t="str">
+        <x:v>Emerging-technology Centres of Excellence under the UP Startup Policy</x:v>
+      </x:c>
+      <x:c r="G137" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H137" t="str">
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+      </x:c>
+      <x:c r="I137" t="str">
+        <x:v>AI/ML, drone, MedTech and emerging-technology startup support</x:v>
+      </x:c>
+      <x:c r="J137" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K137" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L137" t="str">
+        <x:v>AI/ML, drones, MedTech, blockchain, 5G/6G and additive manufacturing</x:v>
+      </x:c>
+      <x:c r="M137" t="str">
+        <x:v>The official StartinUP portal reports established CoEs in AI/ML, drones and MedTech and further planned emerging-tech CoEs.</x:v>
+      </x:c>
+      <x:c r="N137" t="str">
+        <x:v>https://invest.up.gov.in/startup-sector/</x:v>
+      </x:c>
+      <x:c r="O137" t="str"/>
+      <x:c r="P137" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q137" t="str"/>
+      <x:c r="R137" t="str"/>
+      <x:c r="S137" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
     <x:row r="138">
-      <x:c r="A138"/>
-      <x:c r="B138"/>
-      <x:c r="C138"/>
-      <x:c r="D138"/>
-      <x:c r="E138"/>
-      <x:c r="F138"/>
-      <x:c r="G138"/>
-      <x:c r="H138"/>
-      <x:c r="I138"/>
-      <x:c r="J138"/>
-      <x:c r="K138"/>
-      <x:c r="L138"/>
-      <x:c r="M138"/>
-      <x:c r="N138"/>
-      <x:c r="O138"/>
-      <x:c r="P138"/>
-      <x:c r="Q138"/>
-      <x:c r="R138"/>
-      <x:c r="S138"/>
+      <x:c r="A138" t="str">
+        <x:v>ai-137</x:v>
+      </x:c>
+      <x:c r="B138" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>Government of Kerala / KSCSTE</x:v>
+      </x:c>
+      <x:c r="F138" t="str">
+        <x:v>Centre for Artificial Intelligence in Agriculture under Kerala Biotechnology Policy 2026</x:v>
+      </x:c>
+      <x:c r="G138" t="str">
+        <x:v>Agriculture</x:v>
+      </x:c>
+      <x:c r="H138" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I138" t="str">
+        <x:v>Precision agriculture, crop health and pest surveillance</x:v>
+      </x:c>
+      <x:c r="J138" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K138" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L138" t="str">
+        <x:v>Integrated agricultural datasets, AI pest surveillance, weather prediction and irrigation scheduling</x:v>
+      </x:c>
+      <x:c r="M138" t="str">
+        <x:v>The official Kerala Biotechnology Policy 2026 mandates a Centre for AI in Agriculture and lists its operational use cases.</x:v>
+      </x:c>
+      <x:c r="N138" t="str">
+        <x:v>https://kscste.kerala.gov.in/storage/2026/03/KBC_Biotech-Policy_26m.pdf</x:v>
+      </x:c>
+      <x:c r="O138" t="str"/>
+      <x:c r="P138" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q138" t="str"/>
+      <x:c r="R138" t="str"/>
+      <x:c r="S138" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>ai-138</x:v>
+      </x:c>
+      <x:c r="B139" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C139" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D139" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E139" t="str">
+        <x:v>K-DISC / Kerala Genome Data Centre</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>Kerala Genome Data Centre for medical, agricultural and livestock genomics</x:v>
+      </x:c>
+      <x:c r="G139" t="str">
+        <x:v>Healthcare</x:v>
+      </x:c>
+      <x:c r="H139" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I139" t="str">
+        <x:v>Genomic data infrastructure and life-science research</x:v>
+      </x:c>
+      <x:c r="J139" t="str">
+        <x:v>₹150 crore hardware/software + ₹300 crore genomic-data generation; ₹450 crore total</x:v>
+      </x:c>
+      <x:c r="K139" t="str">
+        <x:v>Government programme investment</x:v>
+      </x:c>
+      <x:c r="L139" t="str">
+        <x:v>High-capacity genomic data management, analytics, research datasets and ethical data standards</x:v>
+      </x:c>
+      <x:c r="M139" t="str">
+        <x:v>The official KGDC page states ₹150 crore for hardware/software and ₹300 crore for four years of genomic data generation.</x:v>
+      </x:c>
+      <x:c r="N139" t="str">
+        <x:v>https://kgdc.kerala.gov.in/about/</x:v>
+      </x:c>
+      <x:c r="O139" t="str">
+        <x:v>INR</x:v>
+      </x:c>
+      <x:c r="P139" s="2" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q139" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="R139" t="str"/>
+      <x:c r="S139" t="str">
+        <x:v>Parsed INR crore amount from the cited government source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>ai-139</x:v>
+      </x:c>
+      <x:c r="B140" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C140" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D140" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E140" t="str">
+        <x:v>Government of Kerala / Electronics &amp; IT Department</x:v>
+      </x:c>
+      <x:c r="F140" t="str">
+        <x:v>Ten-year Kerala AI Mission</x:v>
+      </x:c>
+      <x:c r="G140" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H140" t="str">
+        <x:v>AI Strategy &amp; Governance</x:v>
+      </x:c>
+      <x:c r="I140" t="str">
+        <x:v>Ethical AI governance and public-sector modernization</x:v>
+      </x:c>
+      <x:c r="J140" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K140" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L140" t="str">
+        <x:v>State AI governance framework, 50 government AI solutions and responsible adoption</x:v>
+      </x:c>
+      <x:c r="M140" t="str">
+        <x:v>Kerala IT Policy 2026 defines a ten-year AI Mission, 50 governance/PSU solutions and an AI-ready workforce target of 100,000.</x:v>
+      </x:c>
+      <x:c r="N140" t="str">
+        <x:v>https://kfon.kerala.gov.in/wp-content/uploads/2026/02/IT_policy_2026_Kerala.pdf</x:v>
+      </x:c>
+      <x:c r="O140" t="str"/>
+      <x:c r="P140" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q140" t="str"/>
+      <x:c r="R140" t="str"/>
+      <x:c r="S140" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>ai-140</x:v>
+      </x:c>
+      <x:c r="B141" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>Kerala Infrastructure and Technology for Education</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>Responsible AI curriculum and Samagra AI Engine</x:v>
+      </x:c>
+      <x:c r="G141" t="str">
+        <x:v>Education &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="H141" t="str">
+        <x:v>AI Talent &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="I141" t="str">
+        <x:v>School AI curriculum, teacher training and public AI literacy</x:v>
+      </x:c>
+      <x:c r="J141" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K141" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L141" t="str">
+        <x:v>Responsible AI, robotics, prompt engineering, RAG and curriculum-aligned LLM services</x:v>
+      </x:c>
+      <x:c r="M141" t="str">
+        <x:v>The official KITE AI portal documents completed teacher training, AI curriculum from Class 7 and the Samagra AI Engine rollout.</x:v>
+      </x:c>
+      <x:c r="N141" t="str">
+        <x:v>https://ai.kite.kerala.gov.in/</x:v>
+      </x:c>
+      <x:c r="O141" t="str"/>
+      <x:c r="P141" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q141" t="str"/>
+      <x:c r="R141" t="str"/>
+      <x:c r="S141" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
+        <x:v>ai-141</x:v>
+      </x:c>
+      <x:c r="B142" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>Government of Kerala / Digital Science Park</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>Digital Science Park Industry 4.0 and smart-hardware facilities</x:v>
+      </x:c>
+      <x:c r="G142" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H142" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="I142" t="str">
+        <x:v>Industry 4.0, robotics and smart manufacturing</x:v>
+      </x:c>
+      <x:c r="J142" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K142" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L142" t="str">
+        <x:v>Industry 4.0, robotics, smart hardware, 5G and advanced materials</x:v>
+      </x:c>
+      <x:c r="M142" t="str">
+        <x:v>The official Kerala government page describes operational Digital Science Park facilities for Industry 4.0, robotics, electronics and smart hardware.</x:v>
+      </x:c>
+      <x:c r="N142" t="str">
+        <x:v>https://kerala.gov.in/articledetail/NjA0NjQ5MzUxLjI0/0?lan=en</x:v>
+      </x:c>
+      <x:c r="O142" t="str"/>
+      <x:c r="P142" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q142" t="str"/>
+      <x:c r="R142" t="str"/>
+      <x:c r="S142" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>ai-142</x:v>
+      </x:c>
+      <x:c r="B143" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>Thiruvananthapuram</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>Government of Kerala / Digital Science Park</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>AI and deep-tech infrastructure at Digital Science Park</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="H143" t="str">
+        <x:v>Cloud &amp; Compute</x:v>
+      </x:c>
+      <x:c r="I143" t="str">
+        <x:v>AI research compute, high-end data centres and digital deep tech</x:v>
+      </x:c>
+      <x:c r="J143" t="str">
+        <x:v>₹1,515 crore total estimated project outlay</x:v>
+      </x:c>
+      <x:c r="K143" t="str">
+        <x:v>Government project outlay</x:v>
+      </x:c>
+      <x:c r="L143" t="str">
+        <x:v>AI research infrastructure, high-end data centres, 5G, blockchain and cybersecurity labs</x:v>
+      </x:c>
+      <x:c r="M143" t="str">
+        <x:v>The official Kerala government page reports the park's AI/deep-tech scope and ₹1,515 crore total estimated outlay.</x:v>
+      </x:c>
+      <x:c r="N143" t="str">
+        <x:v>https://kerala.gov.in/articledetail/NjA0NjQ5MzUxLjI0/0?lan=en</x:v>
+      </x:c>
+      <x:c r="O143" t="str">
+        <x:v>INR</x:v>
+      </x:c>
+      <x:c r="P143" s="2" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q143" t="n">
+        <x:v>1515</x:v>
+      </x:c>
+      <x:c r="R143" t="str"/>
+      <x:c r="S143" t="str">
+        <x:v>Parsed INR crore amount from the cited government source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>ai-143</x:v>
+      </x:c>
+      <x:c r="B144" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>Kerala State IT Mission</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>K-AI innovation gateway for departmental AI use cases</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I144" t="str">
+        <x:v>Cross-department AI use-case intake and implementation</x:v>
+      </x:c>
+      <x:c r="J144" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K144" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L144" t="str">
+        <x:v>Structured AI idea capture, expert evaluation, implementation monitoring and startup collaboration</x:v>
+      </x:c>
+      <x:c r="M144" t="str">
+        <x:v>The official K-AI portal reports participation by 18 departments, 51 use cases and 237 submitted proposals.</x:v>
+      </x:c>
+      <x:c r="N144" t="str">
+        <x:v>https://kai.kerala.gov.in/</x:v>
+      </x:c>
+      <x:c r="O144" t="str"/>
+      <x:c r="P144" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q144" t="str"/>
+      <x:c r="R144" t="str"/>
+      <x:c r="S144" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>ai-144</x:v>
+      </x:c>
+      <x:c r="B145" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>Government of Kerala / Kerala State IT Mission</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>Kerala AVGC-XR Policy with AI Media focus</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>Marketing &amp; Advertising</x:v>
+      </x:c>
+      <x:c r="H145" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I145" t="str">
+        <x:v>AI-enabled media, animation, VFX, gaming and immersive content</x:v>
+      </x:c>
+      <x:c r="J145" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K145" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L145" t="str">
+        <x:v>AI media, automation, simulation, XR, digital twins and OTT content platforms</x:v>
+      </x:c>
+      <x:c r="M145" t="str">
+        <x:v>The officially approved AVGC-XR policy identifies AI Media and automation as focus areas and targets 250 establishments and 50,000 jobs by 2029.</x:v>
+      </x:c>
+      <x:c r="N145" t="str">
+        <x:v>https://document.kerala.gov.in/documents/cabinetdecisions/cabinet2203202414%3A46%3A24.pdf</x:v>
+      </x:c>
+      <x:c r="O145" t="str"/>
+      <x:c r="P145" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q145" t="str"/>
+      <x:c r="R145" t="str"/>
+      <x:c r="S145" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>ai-145</x:v>
+      </x:c>
+      <x:c r="B146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C146" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>Government of Kerala / Invest Kerala</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>Electronics System Design &amp; Manufacturing ecosystem and Maker Village</x:v>
+      </x:c>
+      <x:c r="G146" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H146" t="str">
+        <x:v>Semiconductor &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="I146" t="str">
+        <x:v>Electronic hardware, chip design and ESDM incubation</x:v>
+      </x:c>
+      <x:c r="J146" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K146" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L146" t="str">
+        <x:v>Electronic system design, semiconductor/electronics skills and hardware prototyping</x:v>
+      </x:c>
+      <x:c r="M146" t="str">
+        <x:v>The official Invest Kerala page documents the state ESDM ecosystem and Maker Village hardware incubator backed by MeitY, IIITM-K and Kerala Startup Mission.</x:v>
+      </x:c>
+      <x:c r="N146" t="str">
+        <x:v>https://www.invest.kerala.gov.in/doing-business-in-kerala/thriving-sectors/electronics-system-design-manufacturing-esdm/</x:v>
+      </x:c>
+      <x:c r="O146" t="str"/>
+      <x:c r="P146" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q146" t="str"/>
+      <x:c r="R146" t="str"/>
+      <x:c r="S146" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>ai-146</x:v>
+      </x:c>
+      <x:c r="B147" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>Kerala Startup Mission</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>Government-backed AI, robotics and semiconductor startup ecosystem</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+      </x:c>
+      <x:c r="I147" t="str">
+        <x:v>AI, edge chips, robotics and enterprise-agent startups</x:v>
+      </x:c>
+      <x:c r="J147" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K147" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L147" t="str">
+        <x:v>AI edge chips, autonomous driving, voice AI, marine robotics and health-tech software</x:v>
+      </x:c>
+      <x:c r="M147" t="str">
+        <x:v>The official Kerala Startup Mission portal profiles supported startups spanning AI chips, autonomous systems, voice AI and robotics.</x:v>
+      </x:c>
+      <x:c r="N147" t="str">
+        <x:v>https://startupmission.kerala.gov.in/</x:v>
+      </x:c>
+      <x:c r="O147" t="str"/>
+      <x:c r="P147" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q147" t="str"/>
+      <x:c r="R147" t="str"/>
+      <x:c r="S147" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>ai-147</x:v>
+      </x:c>
+      <x:c r="B148" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>Kerala</x:v>
+      </x:c>
+      <x:c r="E148" t="str">
+        <x:v>Kerala Motor Vehicles Department</x:v>
+      </x:c>
+      <x:c r="F148" t="str">
+        <x:v>Virtual Check Post digital enforcement platform</x:v>
+      </x:c>
+      <x:c r="G148" t="str">
+        <x:v>Transportation</x:v>
+      </x:c>
+      <x:c r="H148" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I148" t="str">
+        <x:v>Vehicle compliance, road safety and digital enforcement</x:v>
+      </x:c>
+      <x:c r="J148" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K148" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L148" t="str">
+        <x:v>AI-driven real-time monitoring, ANPR, automated violation detection and multi-system data integration</x:v>
+      </x:c>
+      <x:c r="M148" t="str">
+        <x:v>The official MVD Virtual Check Post portal describes AI-driven ANPR enforcement and real-time compliance monitoring.</x:v>
+      </x:c>
+      <x:c r="N148" t="str">
+        <x:v>https://enforcement.mvd.kerala.gov.in/</x:v>
+      </x:c>
+      <x:c r="O148" t="str"/>
+      <x:c r="P148" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q148" t="str"/>
+      <x:c r="R148" t="str"/>
+      <x:c r="S148" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>ai-148</x:v>
+      </x:c>
+      <x:c r="B149" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="E149" t="str">
+        <x:v>Government of Karnataka / Karnataka Digital Economy Mission</x:v>
+      </x:c>
+      <x:c r="F149" t="str">
+        <x:v>AI-enabled inclusive development and public-service delivery</x:v>
+      </x:c>
+      <x:c r="G149" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H149" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I149" t="str">
+        <x:v>Applied AI for state services and inclusive development</x:v>
+      </x:c>
+      <x:c r="J149" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K149" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L149" t="str">
+        <x:v>AI decision support and citizen-service applications</x:v>
+      </x:c>
+      <x:c r="M149" t="str">
+        <x:v>KDEM's official state-budget note places artificial intelligence at the core of inclusive development and governance.</x:v>
+      </x:c>
+      <x:c r="N149" t="str">
+        <x:v>https://karnatakadigital.in/news/state-budget-2026-27-artificial-intelligence-at-the-core-of-inclusive-development-and-governance/</x:v>
+      </x:c>
+      <x:c r="O149" t="str"/>
+      <x:c r="P149" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q149" t="str"/>
+      <x:c r="R149" t="str"/>
+      <x:c r="S149" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>ai-149</x:v>
+      </x:c>
+      <x:c r="B150" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>Bengaluru</x:v>
+      </x:c>
+      <x:c r="E150" t="str">
+        <x:v>Government of Karnataka / Karnataka Digital Economy Mission</x:v>
+      </x:c>
+      <x:c r="F150" t="str">
+        <x:v>Karnataka GCC Policy AI Centre of Excellence</x:v>
+      </x:c>
+      <x:c r="G150" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H150" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I150" t="str">
+        <x:v>AI research, datasets, compute and commercialization</x:v>
+      </x:c>
+      <x:c r="J150" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K150" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L150" t="str">
+        <x:v>AI R&amp;D, shared compute, curated datasets, responsible AI and startup acceleration</x:v>
+      </x:c>
+      <x:c r="M150" t="str">
+        <x:v>The official draft GCC policy proposes a Bengaluru AI Centre of Excellence with hub-and-spoke R&amp;D, compute, datasets and startup support.</x:v>
+      </x:c>
+      <x:c r="N150" t="str">
+        <x:v>https://karnatakadigital.in/wp-content/uploads/2024/11/Draft-KarnatakaGCCPolicy2024-2029-.pdf</x:v>
+      </x:c>
+      <x:c r="O150" t="str"/>
+      <x:c r="P150" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q150" t="str"/>
+      <x:c r="R150" t="str"/>
+      <x:c r="S150" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
+        <x:v>ai-150</x:v>
+      </x:c>
+      <x:c r="B151" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>Government of Karnataka / Karnataka Digital Economy Mission</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>Responsible-AI and GCC ecosystem governance framework</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>AI Strategy &amp; Governance</x:v>
+      </x:c>
+      <x:c r="I151" t="str">
+        <x:v>Responsible AI standards and coordinated state ecosystem development</x:v>
+      </x:c>
+      <x:c r="J151" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K151" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L151" t="str">
+        <x:v>Responsible and ethical AI governance, institutional coordination and policy implementation</x:v>
+      </x:c>
+      <x:c r="M151" t="str">
+        <x:v>The official draft GCC policy embeds responsible and ethical AI within the proposed AI Centre of Excellence and state support framework.</x:v>
+      </x:c>
+      <x:c r="N151" t="str">
+        <x:v>https://karnatakadigital.in/wp-content/uploads/2024/11/Draft-KarnatakaGCCPolicy2024-2029-.pdf</x:v>
+      </x:c>
+      <x:c r="O151" t="str"/>
+      <x:c r="P151" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q151" t="str"/>
+      <x:c r="R151" t="str"/>
+      <x:c r="S151" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>ai-151</x:v>
+      </x:c>
+      <x:c r="B152" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>Bengaluru and regional spokes</x:v>
+      </x:c>
+      <x:c r="E152" t="str">
+        <x:v>Government of Karnataka / Karnataka Digital Economy Mission</x:v>
+      </x:c>
+      <x:c r="F152" t="str">
+        <x:v>Shared AI compute and curated-dataset access through the AI Centre of Excellence</x:v>
+      </x:c>
+      <x:c r="G152" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="H152" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I152" t="str">
+        <x:v>Shared AI data and compute infrastructure</x:v>
+      </x:c>
+      <x:c r="J152" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K152" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L152" t="str">
+        <x:v>Curated datasets, common compute resources and hub-and-spoke access</x:v>
+      </x:c>
+      <x:c r="M152" t="str">
+        <x:v>The official draft GCC policy proposes common compute and curated datasets through an AI Centre of Excellence accessible to ecosystem participants.</x:v>
+      </x:c>
+      <x:c r="N152" t="str">
+        <x:v>https://karnatakadigital.in/wp-content/uploads/2024/11/Draft-KarnatakaGCCPolicy2024-2029-.pdf</x:v>
+      </x:c>
+      <x:c r="O152" t="str"/>
+      <x:c r="P152" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q152" t="str"/>
+      <x:c r="R152" t="str"/>
+      <x:c r="S152" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>ai-152</x:v>
+      </x:c>
+      <x:c r="B153" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>Karnataka</x:v>
+      </x:c>
+      <x:c r="E153" t="str">
+        <x:v>Government of Karnataka / Karnataka Digital Economy Mission</x:v>
+      </x:c>
+      <x:c r="F153" t="str">
+        <x:v>AI Centre of Excellence emerging-technology acceleration programme</x:v>
+      </x:c>
+      <x:c r="G153" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H153" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I153" t="str">
+        <x:v>Next-generation AI experimentation and startup acceleration</x:v>
+      </x:c>
+      <x:c r="J153" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K153" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L153" t="str">
+        <x:v>Advanced AI, responsible AI, shared labs and commercialization support</x:v>
+      </x:c>
+      <x:c r="M153" t="str">
+        <x:v>The official draft GCC policy positions the AI Centre of Excellence as a platform for advanced AI experimentation, innovation and startup acceleration.</x:v>
+      </x:c>
+      <x:c r="N153" t="str">
+        <x:v>https://karnatakadigital.in/wp-content/uploads/2024/11/Draft-KarnatakaGCCPolicy2024-2029-.pdf</x:v>
+      </x:c>
+      <x:c r="O153" t="str"/>
+      <x:c r="P153" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q153" t="str"/>
+      <x:c r="R153" t="str"/>
+      <x:c r="S153" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>ai-153</x:v>
+      </x:c>
+      <x:c r="B154" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>Maharashtra</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>Maharashtra</x:v>
+      </x:c>
+      <x:c r="E154" t="str">
+        <x:v>Government of Maharashtra / Agriculture Department</x:v>
+      </x:c>
+      <x:c r="F154" t="str">
+        <x:v>Agriculture Intelligence and Analytics Innovation Centre</x:v>
+      </x:c>
+      <x:c r="G154" t="str">
+        <x:v>Agriculture</x:v>
+      </x:c>
+      <x:c r="H154" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I154" t="str">
+        <x:v>Applied agricultural AI research and field translation</x:v>
+      </x:c>
+      <x:c r="J154" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K154" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L154" t="str">
+        <x:v>AI analytics, research collaboration, responsible adoption and startup solutions</x:v>
+      </x:c>
+      <x:c r="M154" t="str">
+        <x:v>The official AIAIC portal describes a government-backed centre connecting policy, technology, research institutions, startups and field implementation.</x:v>
+      </x:c>
+      <x:c r="N154" t="str">
+        <x:v>https://aiaic.maharashtra.gov.in/ContentPages/AboutUs.aspx/</x:v>
+      </x:c>
+      <x:c r="O154" t="str"/>
+      <x:c r="P154" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q154" t="str"/>
+      <x:c r="R154" t="str"/>
+      <x:c r="S154" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>ai-154</x:v>
+      </x:c>
+      <x:c r="B155" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>Maharashtra</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>Maharashtra</x:v>
+      </x:c>
+      <x:c r="E155" t="str">
+        <x:v>Electronics, IT and AI Department, Government of Maharashtra</x:v>
+      </x:c>
+      <x:c r="F155" t="str">
+        <x:v>Tech-Saturday statewide digital-capacity programme</x:v>
+      </x:c>
+      <x:c r="G155" t="str">
+        <x:v>Education &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="H155" t="str">
+        <x:v>AI Talent &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="I155" t="str">
+        <x:v>Government workforce capacity for emerging technologies</x:v>
+      </x:c>
+      <x:c r="J155" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K155" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L155" t="str">
+        <x:v>Hands-on emerging-technology training, digital tools and live demonstrations</x:v>
+      </x:c>
+      <x:c r="M155" t="str">
+        <x:v>The department's official page documents a monthly hands-on technology programme for government officers that has expanded to every district.</x:v>
+      </x:c>
+      <x:c r="N155" t="str">
+        <x:v>https://it.maharashtra.gov.in/tech-saturday/</x:v>
+      </x:c>
+      <x:c r="O155" t="str"/>
+      <x:c r="P155" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q155" t="str"/>
+      <x:c r="R155" t="str"/>
+      <x:c r="S155" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>ai-155</x:v>
+      </x:c>
+      <x:c r="B156" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>Telangana</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>Telangana</x:v>
+      </x:c>
+      <x:c r="E156" t="str">
+        <x:v>Government of Telangana / Invest Telangana</x:v>
+      </x:c>
+      <x:c r="F156" t="str">
+        <x:v>Centre for Research in Applied Artificial Intelligence</x:v>
+      </x:c>
+      <x:c r="G156" t="str">
+        <x:v>Healthcare</x:v>
+      </x:c>
+      <x:c r="H156" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I156" t="str">
+        <x:v>Applied AI research in healthcare and mobility</x:v>
+      </x:c>
+      <x:c r="J156" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K156" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L156" t="str">
+        <x:v>Applied AI research, health technology, mobility and industry-academia collaboration</x:v>
+      </x:c>
+      <x:c r="M156" t="str">
+        <x:v>The official Invest Telangana portal describes the applied-AI research centre and its healthcare and mobility focus.</x:v>
+      </x:c>
+      <x:c r="N156" t="str">
+        <x:v>https://invest.telangana.gov.in/emerging-technologies/</x:v>
+      </x:c>
+      <x:c r="O156" t="str"/>
+      <x:c r="P156" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q156" t="str"/>
+      <x:c r="R156" t="str"/>
+      <x:c r="S156" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>ai-156</x:v>
+      </x:c>
+      <x:c r="B157" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>Telangana</x:v>
+      </x:c>
+      <x:c r="D157" t="str">
+        <x:v>Telangana</x:v>
+      </x:c>
+      <x:c r="E157" t="str">
+        <x:v>Government of Telangana</x:v>
+      </x:c>
+      <x:c r="F157" t="str">
+        <x:v>Telangana Rising 2047 AI-enabled GCC and facility-operations programme</x:v>
+      </x:c>
+      <x:c r="G157" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H157" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="I157" t="str">
+        <x:v>Enterprise automation and AI-enabled operational management</x:v>
+      </x:c>
+      <x:c r="J157" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K157" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L157" t="str">
+        <x:v>AI-enabled facility management, enterprise analytics and high-value GCC operations</x:v>
+      </x:c>
+      <x:c r="M157" t="str">
+        <x:v>The official Telangana Rising 2047 strategy calls for AI-enabled facility management and high-value GCC operations across the state economy.</x:v>
+      </x:c>
+      <x:c r="N157" t="str">
+        <x:v>https://tgswc.telangana.gov.in/wp-content/uploads/2025/12/TelanganaRising-2047.pdf</x:v>
+      </x:c>
+      <x:c r="O157" t="str"/>
+      <x:c r="P157" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q157" t="str"/>
+      <x:c r="R157" t="str"/>
+      <x:c r="S157" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>ai-157</x:v>
+      </x:c>
+      <x:c r="B158" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>Telangana</x:v>
+      </x:c>
+      <x:c r="D158" t="str">
+        <x:v>Telangana</x:v>
+      </x:c>
+      <x:c r="E158" t="str">
+        <x:v>ITE&amp;C Department, Government of Telangana</x:v>
+      </x:c>
+      <x:c r="F158" t="str">
+        <x:v>Telangana Data Exchange (TGDeX)</x:v>
+      </x:c>
+      <x:c r="G158" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H158" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I158" t="str">
+        <x:v>Secure government data exchange and reusable AI assets</x:v>
+      </x:c>
+      <x:c r="J158" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K158" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L158" t="str">
+        <x:v>Secure data exchange, sector data banks, reusable AI models and governed access</x:v>
+      </x:c>
+      <x:c r="M158" t="str">
+        <x:v>The official TGDeX portal reports more than 300 data banks and 50 AI models across over 25 sectors for governed public use cases.</x:v>
+      </x:c>
+      <x:c r="N158" t="str">
+        <x:v>https://tgdex.telangana.gov.in/about-us</x:v>
+      </x:c>
+      <x:c r="O158" t="str"/>
+      <x:c r="P158" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q158" t="str"/>
+      <x:c r="R158" t="str"/>
+      <x:c r="S158" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>ai-158</x:v>
+      </x:c>
+      <x:c r="B159" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="E159" t="str">
+        <x:v>Tamil Nadu e-Governance Agency / iTNT Hub</x:v>
+      </x:c>
+      <x:c r="F159" t="str">
+        <x:v>Public Sector Innovation Challenge</x:v>
+      </x:c>
+      <x:c r="G159" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H159" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I159" t="str">
+        <x:v>AI solutions for state problem statements</x:v>
+      </x:c>
+      <x:c r="J159" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K159" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L159" t="str">
+        <x:v>Artificial intelligence, machine learning, cloud services and data sandboxes</x:v>
+      </x:c>
+      <x:c r="M159" t="str">
+        <x:v>The official iTNT Hub challenge invites AI-driven solutions for government problem statements and provides cloud and data-sandbox support.</x:v>
+      </x:c>
+      <x:c r="N159" t="str">
+        <x:v>https://itnthub.tn.gov.in/public_sector%20_nnovation_challenge.html</x:v>
+      </x:c>
+      <x:c r="O159" t="str"/>
+      <x:c r="P159" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q159" t="str"/>
+      <x:c r="R159" t="str"/>
+      <x:c r="S159" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>ai-159</x:v>
+      </x:c>
+      <x:c r="B160" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C160" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="D160" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="E160" t="str">
+        <x:v>Tamil Nadu e-Governance Agency</x:v>
+      </x:c>
+      <x:c r="F160" t="str">
+        <x:v>Tamil Nadu Artificial Intelligence Mission government-adoption programme</x:v>
+      </x:c>
+      <x:c r="G160" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H160" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="I160" t="str">
+        <x:v>Predictive administration and process modernization</x:v>
+      </x:c>
+      <x:c r="J160" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K160" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L160" t="str">
+        <x:v>Predictive analytics, AI-supported decisions and government process automation</x:v>
+      </x:c>
+      <x:c r="M160" t="str">
+        <x:v>The official IT department policy note assigns TNAIM responsibility for predictive policy support and AI adoption across government.</x:v>
+      </x:c>
+      <x:c r="N160" t="str">
+        <x:v>https://tnega.tn.gov.in/assets/pdf/it_e_pn_2025_26.pdf</x:v>
+      </x:c>
+      <x:c r="O160" t="str"/>
+      <x:c r="P160" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q160" t="str"/>
+      <x:c r="R160" t="str"/>
+      <x:c r="S160" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>ai-160</x:v>
+      </x:c>
+      <x:c r="B161" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C161" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="D161" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="E161" t="str">
+        <x:v>Tamil Nadu e-Governance Agency</x:v>
+      </x:c>
+      <x:c r="F161" t="str">
+        <x:v>TNAIM shared compute, storage and data-enablement framework</x:v>
+      </x:c>
+      <x:c r="G161" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="H161" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I161" t="str">
+        <x:v>Shared AI compute, storage and public-sector data enablement</x:v>
+      </x:c>
+      <x:c r="J161" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K161" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L161" t="str">
+        <x:v>AI compute, storage, data access and common mission infrastructure</x:v>
+      </x:c>
+      <x:c r="M161" t="str">
+        <x:v>The official IT department policy note includes compute and storage enablement within the Tamil Nadu Artificial Intelligence Mission.</x:v>
+      </x:c>
+      <x:c r="N161" t="str">
+        <x:v>https://tnega.tn.gov.in/assets/pdf/it_e_pn_2025_26.pdf</x:v>
+      </x:c>
+      <x:c r="O161" t="str"/>
+      <x:c r="P161" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q161" t="str"/>
+      <x:c r="R161" t="str"/>
+      <x:c r="S161" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>ai-161</x:v>
+      </x:c>
+      <x:c r="B162" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C162" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="D162" t="str">
+        <x:v>Tamil Nadu</x:v>
+      </x:c>
+      <x:c r="E162" t="str">
+        <x:v>Tamil Nadu e-Governance Agency / iTNT Hub</x:v>
+      </x:c>
+      <x:c r="F162" t="str">
+        <x:v>TNAIM emerging-AI innovation and startup programme</x:v>
+      </x:c>
+      <x:c r="G162" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H162" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I162" t="str">
+        <x:v>Emerging AI pilots, innovation challenges and startup support</x:v>
+      </x:c>
+      <x:c r="J162" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K162" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L162" t="str">
+        <x:v>Advanced AI pilots, innovation sandboxes and startup-led public-sector solutions</x:v>
+      </x:c>
+      <x:c r="M162" t="str">
+        <x:v>The official policy note and iTNT delivery platform position TNAIM to support AI innovation, startups and mission-led pilots.</x:v>
+      </x:c>
+      <x:c r="N162" t="str">
+        <x:v>https://tnega.tn.gov.in/assets/pdf/it_e_pn_2025_26.pdf</x:v>
+      </x:c>
+      <x:c r="O162" t="str"/>
+      <x:c r="P162" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q162" t="str"/>
+      <x:c r="R162" t="str"/>
+      <x:c r="S162" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" t="str">
+        <x:v>ai-162</x:v>
+      </x:c>
+      <x:c r="B163" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C163" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="D163" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="E163" t="str">
+        <x:v>Department of Science and Technology, Government of Gujarat</x:v>
+      </x:c>
+      <x:c r="F163" t="str">
+        <x:v>Gujarat AI Innovation Challenge</x:v>
+      </x:c>
+      <x:c r="G163" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H163" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="I163" t="str">
+        <x:v>Government AI use-case pilots and production rollouts</x:v>
+      </x:c>
+      <x:c r="J163" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K163" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L163" t="str">
+        <x:v>AI proofs of concept, evaluation sandboxes and production-scale public-service solutions</x:v>
+      </x:c>
+      <x:c r="M163" t="str">
+        <x:v>The official government resolution establishes a structured AI Innovation Challenge for selecting, funding and scaling departmental use cases.</x:v>
+      </x:c>
+      <x:c r="N163" t="str">
+        <x:v>https://dst.gujarat.gov.in/ViewFile?fileName=0ryyfossIfrnK3nTSB6DigDNC8sV7UEe%E2%9C%A4Bs244MkMaQXivO2UR0ZGWpek1G3wLvJ%E2%9C%BFtcvcaPnnJPErYpE6nxryem1F%E2%9C%A4wwdcshGvAXdLdMfxp%E2%9C%A49jF0K4K2fGW%E2%9C%A4k4Fa%E2%9C%A4kswYrHNG%E2%9C%A4%E2%9C%BFruhnIdXzXDdGDfg%E2%99%AC%E2%99%AC</x:v>
+      </x:c>
+      <x:c r="O163" t="str"/>
+      <x:c r="P163" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q163" t="str"/>
+      <x:c r="R163" t="str"/>
+      <x:c r="S163" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>ai-163</x:v>
+      </x:c>
+      <x:c r="B164" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C164" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="E164" t="str">
+        <x:v>Department of Science and Technology, Government of Gujarat</x:v>
+      </x:c>
+      <x:c r="F164" t="str">
+        <x:v>Viksit Gujarat API-based performance-monitoring framework</x:v>
+      </x:c>
+      <x:c r="G164" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H164" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="I164" t="str">
+        <x:v>Automated programme monitoring and administrative analytics</x:v>
+      </x:c>
+      <x:c r="J164" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K164" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L164" t="str">
+        <x:v>API-based integration, automated KPI monitoring and executive dashboards</x:v>
+      </x:c>
+      <x:c r="M164" t="str">
+        <x:v>The official Viksit Gujarat strategy document specifies API-driven data integration and automated KPI monitoring for programme execution.</x:v>
+      </x:c>
+      <x:c r="N164" t="str">
+        <x:v>https://dst.gujarat.gov.in/ViewFile?fileName=59n4CHE8hT5O9e1bY15gKteAbAHYP4%E2%9C%A4ONIjAc2MHpteSUzlxriaCckr6LIuX5NCLZ%E2%9C%BFaW1NMtPzNhzUQ47Bh0%E2%9C%BF8%E2%9C%A4eS4Y%E2%9C%BFp%E2%9C%BFSJbfPD2VNPc4%E2%9C%A4WDZoy5c71xOC3KCYZKu7Gah9u5MgeF3S2RYV5nykyoA%E2%99%AC%E2%99%AC</x:v>
+      </x:c>
+      <x:c r="O164" t="str"/>
+      <x:c r="P164" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q164" t="str"/>
+      <x:c r="R164" t="str"/>
+      <x:c r="S164" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>ai-164</x:v>
+      </x:c>
+      <x:c r="B165" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C165" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="D165" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="E165" t="str">
+        <x:v>Department of Science and Technology, Government of Gujarat</x:v>
+      </x:c>
+      <x:c r="F165" t="str">
+        <x:v>Gujarat State Data Governance Framework</x:v>
+      </x:c>
+      <x:c r="G165" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H165" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I165" t="str">
+        <x:v>Secure cross-government data exchange and governance</x:v>
+      </x:c>
+      <x:c r="J165" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K165" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L165" t="str">
+        <x:v>Governed data exchange supporting AI, blockchain, IoT and edge-computing use cases</x:v>
+      </x:c>
+      <x:c r="M165" t="str">
+        <x:v>The official framework defines secure data sharing across government entities to support AI and other emerging-technology services.</x:v>
+      </x:c>
+      <x:c r="N165" t="str">
+        <x:v>https://dst.gujarat.gov.in/dst/ViewFile?fileName=EqJ2TlVJgYTCNGhOgjP77hHfmUYD00%E2%9C%BFG%E2%9C%BFnl9KC449JTUEEZNfc6K8dw1mvrIkTES%E2%9C%BFvPdFIwqSygKRrDu5P9EXZiSUXOpuE2TfMB5Y93aKiwrlg2ySmzGmRLUpD%E2%9C%BFGzGMAf5XiUSI7jqTi%E2%9C%BFhIHi13QDQ%E2%99%AC%E2%99%AC</x:v>
+      </x:c>
+      <x:c r="O165" t="str"/>
+      <x:c r="P165" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q165" t="str"/>
+      <x:c r="R165" t="str"/>
+      <x:c r="S165" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>ai-165</x:v>
+      </x:c>
+      <x:c r="B166" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C166" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="D166" t="str">
+        <x:v>Gujarat</x:v>
+      </x:c>
+      <x:c r="E166" t="str">
+        <x:v>Department of Science and Technology, Government of Gujarat</x:v>
+      </x:c>
+      <x:c r="F166" t="str">
+        <x:v>Gujarat Science, Technology and Innovation Policy 2026-31</x:v>
+      </x:c>
+      <x:c r="G166" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H166" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I166" t="str">
+        <x:v>Frontier technology research and innovation ecosystem</x:v>
+      </x:c>
+      <x:c r="J166" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K166" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L166" t="str">
+        <x:v>Artificial intelligence, semiconductors, quantum technologies and advanced research infrastructure</x:v>
+      </x:c>
+      <x:c r="M166" t="str">
+        <x:v>The official STI policy portal identifies AI and other frontier technologies as priority areas for research talent and innovation-system development.</x:v>
+      </x:c>
+      <x:c r="N166" t="str">
+        <x:v>https://dst.gujarat.gov.in/Home/stip</x:v>
+      </x:c>
+      <x:c r="O166" t="str"/>
+      <x:c r="P166" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q166" t="str"/>
+      <x:c r="R166" t="str"/>
+      <x:c r="S166" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>ai-166</x:v>
+      </x:c>
+      <x:c r="B167" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C167" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="D167" t="str">
+        <x:v>Gurugram and Panchkula</x:v>
+      </x:c>
+      <x:c r="E167" t="str">
+        <x:v>Government of Haryana</x:v>
+      </x:c>
+      <x:c r="F167" t="str">
+        <x:v>Global AI Centre and Haryana Advanced Computing Facility</x:v>
+      </x:c>
+      <x:c r="G167" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H167" t="str">
+        <x:v>AI Research &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="I167" t="str">
+        <x:v>AI research, innovation and advanced-computing capacity</x:v>
+      </x:c>
+      <x:c r="J167" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K167" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L167" t="str">
+        <x:v>Applied AI R&amp;D, advanced computing, industry-academia collaboration and shared facilities</x:v>
+      </x:c>
+      <x:c r="M167" t="str">
+        <x:v>The official Make in Haryana Industrial Policy identifies the two facilities for AI research, innovation and capacity building.</x:v>
+      </x:c>
+      <x:c r="N167" t="str">
+        <x:v>https://investharyana.in/content/pdfs/Make%20in%20Haryana%20Industrial%20Policy%202025%20-%2015.09.2025.pdf</x:v>
+      </x:c>
+      <x:c r="O167" t="str"/>
+      <x:c r="P167" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q167" t="str"/>
+      <x:c r="R167" t="str"/>
+      <x:c r="S167" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" t="str">
+        <x:v>ai-167</x:v>
+      </x:c>
+      <x:c r="B168" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C168" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="D168" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="E168" t="str">
+        <x:v>Government of Haryana</x:v>
+      </x:c>
+      <x:c r="F168" t="str">
+        <x:v>Haryana AI Development Programme</x:v>
+      </x:c>
+      <x:c r="G168" t="str">
+        <x:v>Government &amp; Public Services</x:v>
+      </x:c>
+      <x:c r="H168" t="str">
+        <x:v>AI Strategy &amp; Governance</x:v>
+      </x:c>
+      <x:c r="I168" t="str">
+        <x:v>Coordinated statewide AI ecosystem and adoption programme</x:v>
+      </x:c>
+      <x:c r="J168" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K168" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L168" t="str">
+        <x:v>AI programme governance, institutional coordination and capacity development</x:v>
+      </x:c>
+      <x:c r="M168" t="str">
+        <x:v>The official industrial policy sets out the Haryana AI Development Programme alongside dedicated AI and advanced-computing institutions.</x:v>
+      </x:c>
+      <x:c r="N168" t="str">
+        <x:v>https://investharyana.in/content/pdfs/Make%20in%20Haryana%20Industrial%20Policy%202025%20-%2015.09.2025.pdf</x:v>
+      </x:c>
+      <x:c r="O168" t="str"/>
+      <x:c r="P168" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q168" t="str"/>
+      <x:c r="R168" t="str"/>
+      <x:c r="S168" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" t="str">
+        <x:v>ai-168</x:v>
+      </x:c>
+      <x:c r="B169" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C169" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="D169" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="E169" t="str">
+        <x:v>Government of Haryana</x:v>
+      </x:c>
+      <x:c r="F169" t="str">
+        <x:v>Sectoral Centres of Excellence in AI and AVGC-XR</x:v>
+      </x:c>
+      <x:c r="G169" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H169" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I169" t="str">
+        <x:v>Emerging-technology labs and industry-linked centres</x:v>
+      </x:c>
+      <x:c r="J169" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K169" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L169" t="str">
+        <x:v>Artificial intelligence, AVGC-XR and advanced digital-production technologies</x:v>
+      </x:c>
+      <x:c r="M169" t="str">
+        <x:v>The official industrial policy provides for sectoral Centres of Excellence covering AI, AVGC-XR and other emerging industries.</x:v>
+      </x:c>
+      <x:c r="N169" t="str">
+        <x:v>https://investharyana.in/content/pdfs/Make%20in%20Haryana%20Industrial%20Policy%202025%20-%2015.09.2025.pdf</x:v>
+      </x:c>
+      <x:c r="O169" t="str"/>
+      <x:c r="P169" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q169" t="str"/>
+      <x:c r="R169" t="str"/>
+      <x:c r="S169" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" t="str">
+        <x:v>ai-169</x:v>
+      </x:c>
+      <x:c r="B170" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C170" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="D170" t="str">
+        <x:v>Haryana</x:v>
+      </x:c>
+      <x:c r="E170" t="str">
+        <x:v>Government of Haryana</x:v>
+      </x:c>
+      <x:c r="F170" t="str">
+        <x:v>Electronics Centre of Excellence support under Make in Haryana</x:v>
+      </x:c>
+      <x:c r="G170" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H170" t="str">
+        <x:v>Semiconductor &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="I170" t="str">
+        <x:v>Electronics R&amp;D, prototyping and industry skills</x:v>
+      </x:c>
+      <x:c r="J170" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K170" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L170" t="str">
+        <x:v>Electronics engineering, shared testing infrastructure and industry-oriented research</x:v>
+      </x:c>
+      <x:c r="M170" t="str">
+        <x:v>The official industrial policy includes Electronics among the priority sectoral Centres of Excellence eligible for state support.</x:v>
+      </x:c>
+      <x:c r="N170" t="str">
+        <x:v>https://investharyana.in/content/pdfs/Make%20in%20Haryana%20Industrial%20Policy%202025%20-%2015.09.2025.pdf</x:v>
+      </x:c>
+      <x:c r="O170" t="str"/>
+      <x:c r="P170" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q170" t="str"/>
+      <x:c r="R170" t="str"/>
+      <x:c r="S170" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>ai-170</x:v>
+      </x:c>
+      <x:c r="B171" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C171" t="str">
+        <x:v>Delhi</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>New Delhi</x:v>
+      </x:c>
+      <x:c r="E171" t="str">
+        <x:v>National Informatics Centre / Government of India</x:v>
+      </x:c>
+      <x:c r="F171" t="str">
+        <x:v>National Data Centre cloud services in Delhi</x:v>
+      </x:c>
+      <x:c r="G171" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="H171" t="str">
+        <x:v>Cloud &amp; Compute</x:v>
+      </x:c>
+      <x:c r="I171" t="str">
+        <x:v>Government cloud and national data-centre capacity</x:v>
+      </x:c>
+      <x:c r="J171" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K171" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L171" t="str">
+        <x:v>Government cloud, shared compute, hosting and resilient digital infrastructure</x:v>
+      </x:c>
+      <x:c r="M171" t="str">
+        <x:v>An official PIB government document identifies the National Data Centre in Delhi as part of NIC's cloud and hosting infrastructure for government.</x:v>
+      </x:c>
+      <x:c r="N171" t="str">
+        <x:v>https://static.pib.gov.in/WriteReadData/specificdocs/documents/2026/feb/doc2026212786901.pdf</x:v>
+      </x:c>
+      <x:c r="O171" t="str"/>
+      <x:c r="P171" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q171" t="str"/>
+      <x:c r="R171" t="str"/>
+      <x:c r="S171" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>ai-171</x:v>
+      </x:c>
+      <x:c r="B172" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C172" t="str">
+        <x:v>Delhi</x:v>
+      </x:c>
+      <x:c r="D172" t="str">
+        <x:v>Delhi</x:v>
+      </x:c>
+      <x:c r="E172" t="str">
+        <x:v>Finance Department, Government of NCT of Delhi</x:v>
+      </x:c>
+      <x:c r="F172" t="str">
+        <x:v>Faceless GST administration using AI, analytics and automation</x:v>
+      </x:c>
+      <x:c r="G172" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="H172" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="I172" t="str">
+        <x:v>Digital tax administration and interoperable compliance analytics</x:v>
+      </x:c>
+      <x:c r="J172" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K172" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L172" t="str">
+        <x:v>Artificial intelligence, data analytics, automated risk assessment and faceless workflows</x:v>
+      </x:c>
+      <x:c r="M172" t="str">
+        <x:v>The official Delhi budget speech describes collaboration on data analytics, automation and AI for faceless tax administration.</x:v>
+      </x:c>
+      <x:c r="N172" t="str">
+        <x:v>https://finance.delhi.gov.in/sites/default/files/Finance/marquee-files/budget_speech_2024-25_english.pdf</x:v>
+      </x:c>
+      <x:c r="O172" t="str"/>
+      <x:c r="P172" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q172" t="str"/>
+      <x:c r="R172" t="str"/>
+      <x:c r="S172" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" t="str">
+        <x:v>ai-172</x:v>
+      </x:c>
+      <x:c r="B173" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C173" t="str">
+        <x:v>Delhi</x:v>
+      </x:c>
+      <x:c r="D173" t="str">
+        <x:v>Delhi</x:v>
+      </x:c>
+      <x:c r="E173" t="str">
+        <x:v>Planning Department, Government of NCT of Delhi</x:v>
+      </x:c>
+      <x:c r="F173" t="str">
+        <x:v>Frontier-technology industrial development focus</x:v>
+      </x:c>
+      <x:c r="G173" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="H173" t="str">
+        <x:v>Emerging AI Capability</x:v>
+      </x:c>
+      <x:c r="I173" t="str">
+        <x:v>AI, robotics and other frontier-technology industries</x:v>
+      </x:c>
+      <x:c r="J173" t="str">
+        <x:v>Not separately disclosed by the cited government source</x:v>
+      </x:c>
+      <x:c r="K173" t="str">
+        <x:v>Government policy / programme</x:v>
+      </x:c>
+      <x:c r="L173" t="str">
+        <x:v>Artificial intelligence, robotics, biotechnology and green technologies</x:v>
+      </x:c>
+      <x:c r="M173" t="str">
+        <x:v>The official Delhi Economic Survey identifies frontier technologies including AI and robotics as a focus for industrial development.</x:v>
+      </x:c>
+      <x:c r="N173" t="str">
+        <x:v>https://delhiplanning.delhi.gov.in/sites/default/files/2026-03/economic_survey_english_0.pdf</x:v>
+      </x:c>
+      <x:c r="O173" t="str"/>
+      <x:c r="P173" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q173" t="str"/>
+      <x:c r="R173" t="str"/>
+      <x:c r="S173" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>ai-173</x:v>
+      </x:c>
+      <x:c r="B174" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C174" t="str">
+        <x:v>Delhi</x:v>
+      </x:c>
+      <x:c r="D174" t="str">
+        <x:v>Delhi Technological University</x:v>
+      </x:c>
+      <x:c r="E174" t="str">
+        <x:v>Delhi Technological University</x:v>
+      </x:c>
+      <x:c r="F174" t="str">
+        <x:v>Vinod Dham Centre of Excellence for Semiconductors and Microelectronics</x:v>
+      </x:c>
+      <x:c r="G174" t="str">
+        <x:v>Manufacturing &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="H174" t="str">
+        <x:v>Semiconductor &amp; Electronics</x:v>
+      </x:c>
+      <x:c r="I174" t="str">
+        <x:v>Semiconductor research, IC manufacturing and workforce development</x:v>
+      </x:c>
+      <x:c r="J174" t="str">
+        <x:v>₹1 crore philanthropic contribution to establish the centre; not government investment</x:v>
+      </x:c>
+      <x:c r="K174" t="str">
+        <x:v>Public-university centre with philanthropic funding</x:v>
+      </x:c>
+      <x:c r="L174" t="str">
+        <x:v>Semiconductor technology, integrated-circuit manufacturing, microelectronics and chip-design R&amp;D</x:v>
+      </x:c>
+      <x:c r="M174" t="str">
+        <x:v>DTU's official centre page records the May 2023 establishment of VDSemiX for semiconductor research, training, innovation and startups.</x:v>
+      </x:c>
+      <x:c r="N174" t="str">
+        <x:v>https://dtu.ac.in/Web/Departments/VinodDhamCenter/index.html</x:v>
+      </x:c>
+      <x:c r="O174" t="str"/>
+      <x:c r="P174" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q174" t="str"/>
+      <x:c r="R174" t="str"/>
+      <x:c r="S174" t="str">
+        <x:v>Excluded because the cited government source does not disclose a separate row-specific financial commitment.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7764,23 +10374,23 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="23.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13.109999656677246" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24.25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.75" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
-      <x:c r="A1" s="23" t="str">
+      <x:c r="A1" s="27" t="str">
         <x:v>Industry</x:v>
       </x:c>
-      <x:c r="B1" s="24" t="str">
+      <x:c r="B1" s="28" t="str">
         <x:v>Capability</x:v>
       </x:c>
-      <x:c r="C1" s="24" t="str">
+      <x:c r="C1" s="28" t="str">
         <x:v>Record Count</x:v>
       </x:c>
-      <x:c r="D1" s="24" t="str">
+      <x:c r="D1" s="28" t="str">
         <x:v>Chartable Count</x:v>
       </x:c>
     </x:row>
@@ -7789,10 +10399,10 @@
         <x:v>Agriculture</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>AI Strategy &amp; Governance</x:v>
+        <x:v>AI Applications</x:v>
       </x:c>
       <x:c r="C2" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D2" s="9" t="n">
         <x:v>0</x:v>
@@ -7803,7 +10413,7 @@
         <x:v>Agriculture</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Emerging AI Capability</x:v>
+        <x:v>AI Research &amp; Innovation</x:v>
       </x:c>
       <x:c r="C3" s="9" t="n">
         <x:v>1</x:v>
@@ -7817,21 +10427,21 @@
         <x:v>Agriculture</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+        <x:v>AI Strategy &amp; Governance</x:v>
       </x:c>
       <x:c r="C4" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D4" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
-        <x:v>Defence &amp; Aerospace</x:v>
+        <x:v>Agriculture</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>Automation &amp; Enterprise Tech</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C5" s="9" t="n">
         <x:v>1</x:v>
@@ -7842,10 +10452,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
-        <x:v>Defence &amp; Aerospace</x:v>
+        <x:v>Agriculture</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>Cloud &amp; Compute</x:v>
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
       </x:c>
       <x:c r="C6" s="9" t="n">
         <x:v>1</x:v>
@@ -7859,13 +10469,13 @@
         <x:v>Defence &amp; Aerospace</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>Emerging AI Capability</x:v>
+        <x:v>AI Research &amp; Innovation</x:v>
       </x:c>
       <x:c r="C7" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -7873,13 +10483,13 @@
         <x:v>Defence &amp; Aerospace</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Semiconductor &amp; Electronics</x:v>
+        <x:v>Automation &amp; Enterprise Tech</x:v>
       </x:c>
       <x:c r="C8" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7887,7 +10497,7 @@
         <x:v>Defence &amp; Aerospace</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+        <x:v>Cloud &amp; Compute</x:v>
       </x:c>
       <x:c r="C9" s="9" t="n">
         <x:v>1</x:v>
@@ -7898,41 +10508,41 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
-        <x:v>Education &amp; Skilling</x:v>
+        <x:v>Defence &amp; Aerospace</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>AI Talent &amp; Skilling</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C10" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D10" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
-        <x:v>Education &amp; Skilling</x:v>
+        <x:v>Defence &amp; Aerospace</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+        <x:v>Semiconductor &amp; Electronics</x:v>
       </x:c>
       <x:c r="C11" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D11" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Defence &amp; Aerospace</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>AI Strategy &amp; Governance</x:v>
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
       </x:c>
       <x:c r="C12" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="9" t="n">
         <x:v>1</x:v>
@@ -7940,30 +10550,30 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Education &amp; Skilling</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>Cloud &amp; Compute</x:v>
+        <x:v>AI Talent &amp; Skilling</x:v>
       </x:c>
       <x:c r="C13" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D13" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Education &amp; Skilling</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str">
-        <x:v>Digital Public Infrastructure</x:v>
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
       </x:c>
       <x:c r="C14" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D14" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -7971,10 +10581,10 @@
         <x:v>Finance</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>Emerging AI Capability</x:v>
+        <x:v>AI Strategy &amp; Governance</x:v>
       </x:c>
       <x:c r="C15" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D15" s="9" t="n">
         <x:v>1</x:v>
@@ -7982,55 +10592,55 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
-        <x:v>Government &amp; Public Services</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>AI Applications</x:v>
+        <x:v>Automation &amp; Enterprise Tech</x:v>
       </x:c>
       <x:c r="C16" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D16" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
-        <x:v>Government &amp; Public Services</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str">
-        <x:v>AI Research &amp; Innovation</x:v>
+        <x:v>Cloud &amp; Compute</x:v>
       </x:c>
       <x:c r="C17" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D17" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
-        <x:v>Government &amp; Public Services</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>AI Strategy &amp; Governance</x:v>
+        <x:v>Digital Public Infrastructure</x:v>
       </x:c>
       <x:c r="C18" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D18" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
-        <x:v>Government &amp; Public Services</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>Digital Public Infrastructure</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C19" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D19" s="9" t="n">
         <x:v>1</x:v>
@@ -8041,13 +10651,13 @@
         <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>Emerging AI Capability</x:v>
+        <x:v>AI Applications</x:v>
       </x:c>
       <x:c r="C20" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D20" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -8055,66 +10665,66 @@
         <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B21" s="9" t="str">
-        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+        <x:v>AI Research &amp; Innovation</x:v>
       </x:c>
       <x:c r="C21" s="9" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D21" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="8" t="str">
-        <x:v>Healthcare</x:v>
+        <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B22" s="9" t="str">
-        <x:v>AI Applications</x:v>
+        <x:v>AI Strategy &amp; Governance</x:v>
       </x:c>
       <x:c r="C22" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D22" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="8" t="str">
-        <x:v>Healthcare</x:v>
+        <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>AI Research &amp; Innovation</x:v>
+        <x:v>Automation &amp; Enterprise Tech</x:v>
       </x:c>
       <x:c r="C23" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D23" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="8" t="str">
-        <x:v>Healthcare</x:v>
+        <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>AI Strategy &amp; Governance</x:v>
+        <x:v>Digital Public Infrastructure</x:v>
       </x:c>
       <x:c r="C24" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D24" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="8" t="str">
-        <x:v>Healthcare</x:v>
+        <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>AI Talent &amp; Skilling</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C25" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D25" s="9" t="n">
         <x:v>1</x:v>
@@ -8122,16 +10732,16 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="8" t="str">
-        <x:v>Healthcare</x:v>
+        <x:v>Government &amp; Public Services</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>Emerging AI Capability</x:v>
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
       </x:c>
       <x:c r="C26" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D26" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -8139,13 +10749,13 @@
         <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>Semiconductor &amp; Electronics</x:v>
+        <x:v>AI Applications</x:v>
       </x:c>
       <x:c r="C27" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D27" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -8153,49 +10763,49 @@
         <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+        <x:v>AI Research &amp; Innovation</x:v>
       </x:c>
       <x:c r="C28" s="9" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="D28" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="8" t="str">
-        <x:v>Manufacturing &amp; Electronics</x:v>
+        <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>Cloud &amp; Compute</x:v>
+        <x:v>AI Strategy &amp; Governance</x:v>
       </x:c>
       <x:c r="C29" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D29" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="8" t="str">
-        <x:v>Manufacturing &amp; Electronics</x:v>
+        <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B30" s="9" t="str">
-        <x:v>Semiconductor &amp; Electronics</x:v>
+        <x:v>AI Talent &amp; Skilling</x:v>
       </x:c>
       <x:c r="C30" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D30" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="8" t="str">
-        <x:v>Marketing &amp; Advertising</x:v>
+        <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B31" s="9" t="str">
-        <x:v>Automation &amp; Enterprise Tech</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C31" s="9" t="n">
         <x:v>1</x:v>
@@ -8206,10 +10816,10 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="8" t="str">
-        <x:v>Technology &amp; Innovation</x:v>
+        <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B32" s="9" t="str">
-        <x:v>AI Research &amp; Innovation</x:v>
+        <x:v>Semiconductor &amp; Electronics</x:v>
       </x:c>
       <x:c r="C32" s="9" t="n">
         <x:v>1</x:v>
@@ -8220,21 +10830,21 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="8" t="str">
-        <x:v>Technology &amp; Innovation</x:v>
+        <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B33" s="9" t="str">
         <x:v>Startup &amp; Innovation Ecosystem</x:v>
       </x:c>
       <x:c r="C33" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D33" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="8" t="str">
-        <x:v>Technology Infrastructure</x:v>
+        <x:v>Manufacturing &amp; Electronics</x:v>
       </x:c>
       <x:c r="B34" s="9" t="str">
         <x:v>Automation &amp; Enterprise Tech</x:v>
@@ -8243,74 +10853,74 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D34" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="8" t="str">
-        <x:v>Technology Infrastructure</x:v>
+        <x:v>Manufacturing &amp; Electronics</x:v>
       </x:c>
       <x:c r="B35" s="9" t="str">
         <x:v>Cloud &amp; Compute</x:v>
       </x:c>
       <x:c r="C35" s="9" t="n">
-        <x:v>21</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D35" s="9" t="n">
-        <x:v>17</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="8" t="str">
-        <x:v>Transportation</x:v>
+        <x:v>Manufacturing &amp; Electronics</x:v>
       </x:c>
       <x:c r="B36" s="9" t="str">
-        <x:v>AI Applications</x:v>
+        <x:v>Semiconductor &amp; Electronics</x:v>
       </x:c>
       <x:c r="C36" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D36" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="8" t="str">
-        <x:v>Transportation</x:v>
+        <x:v>Marketing &amp; Advertising</x:v>
       </x:c>
       <x:c r="B37" s="9" t="str">
-        <x:v>AI Strategy &amp; Governance</x:v>
+        <x:v>Automation &amp; Enterprise Tech</x:v>
       </x:c>
       <x:c r="C37" s="9" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D37" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="8" t="str">
-        <x:v>Transportation</x:v>
+        <x:v>Marketing &amp; Advertising</x:v>
       </x:c>
       <x:c r="B38" s="9" t="str">
-        <x:v>AI Talent &amp; Skilling</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C38" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D38" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="8" t="str">
-        <x:v>Transportation</x:v>
+        <x:v>Technology &amp; Innovation</x:v>
       </x:c>
       <x:c r="B39" s="9" t="str">
-        <x:v>Automation &amp; Enterprise Tech</x:v>
+        <x:v>AI Research &amp; Innovation</x:v>
       </x:c>
       <x:c r="C39" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D39" s="9" t="n">
         <x:v>1</x:v>
@@ -8318,43 +10928,157 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="8" t="str">
-        <x:v>Transportation</x:v>
+        <x:v>Technology &amp; Innovation</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
-        <x:v>Cloud &amp; Compute</x:v>
+        <x:v>Emerging AI Capability</x:v>
       </x:c>
       <x:c r="C40" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D40" s="9" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="8" t="str">
+        <x:v>Technology &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="B41" s="9" t="str">
+        <x:v>Startup &amp; Innovation Ecosystem</x:v>
+      </x:c>
+      <x:c r="C41" s="9" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D41" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="8" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="B42" s="9" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="C42" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D42" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="8" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="B43" s="9" t="str">
+        <x:v>Cloud &amp; Compute</x:v>
+      </x:c>
+      <x:c r="C43" s="9" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D43" s="9" t="n">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="8" t="str">
+        <x:v>Technology Infrastructure</x:v>
+      </x:c>
+      <x:c r="B44" s="9" t="str">
+        <x:v>Digital Public Infrastructure</x:v>
+      </x:c>
+      <x:c r="C44" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D44" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="8" t="str">
         <x:v>Transportation</x:v>
       </x:c>
-      <x:c r="B41" s="9" t="str">
+      <x:c r="B45" s="9" t="str">
+        <x:v>AI Applications</x:v>
+      </x:c>
+      <x:c r="C45" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D45" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="8" t="str">
+        <x:v>Transportation</x:v>
+      </x:c>
+      <x:c r="B46" s="9" t="str">
+        <x:v>AI Strategy &amp; Governance</x:v>
+      </x:c>
+      <x:c r="C46" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D46" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="8" t="str">
+        <x:v>Transportation</x:v>
+      </x:c>
+      <x:c r="B47" s="9" t="str">
+        <x:v>AI Talent &amp; Skilling</x:v>
+      </x:c>
+      <x:c r="C47" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D47" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="8" t="str">
+        <x:v>Transportation</x:v>
+      </x:c>
+      <x:c r="B48" s="9" t="str">
+        <x:v>Automation &amp; Enterprise Tech</x:v>
+      </x:c>
+      <x:c r="C48" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D48" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="8" t="str">
+        <x:v>Transportation</x:v>
+      </x:c>
+      <x:c r="B49" s="9" t="str">
+        <x:v>Cloud &amp; Compute</x:v>
+      </x:c>
+      <x:c r="C49" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D49" s="9" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="8" t="str">
+        <x:v>Transportation</x:v>
+      </x:c>
+      <x:c r="B50" s="9" t="str">
         <x:v>Semiconductor &amp; Electronics</x:v>
       </x:c>
-      <x:c r="C41" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D41" s="9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="8"/>
-      <x:c r="B42" s="9"/>
-      <x:c r="C42" s="9"/>
-      <x:c r="D42" s="10"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="11"/>
-      <x:c r="B43" s="12"/>
-      <x:c r="C43" s="12"/>
-      <x:c r="D43" s="13"/>
+      <x:c r="C50" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D50" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8365,23 +11089,23 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="47.560001373291016" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="184.55999755859375" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="49.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="188.6300048828125" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.3799991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
-      <x:c r="A1" s="23" t="str">
+      <x:c r="A1" s="27" t="str">
         <x:v>Metric</x:v>
       </x:c>
-      <x:c r="B1" s="24" t="str">
+      <x:c r="B1" s="28" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="C1" s="24" t="str">
+      <x:c r="C1" s="28" t="str">
         <x:v>Detail</x:v>
       </x:c>
-      <x:c r="D1" s="24" t="str">
+      <x:c r="D1" s="28" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -8390,7 +11114,7 @@
         <x:v>Records</x:v>
       </x:c>
       <x:c r="B2" s="9" t="n">
-        <x:v>116</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
         <x:v>All rows in Records sheet</x:v>
@@ -8402,7 +11126,7 @@
         <x:v>Chartable records</x:v>
       </x:c>
       <x:c r="B3" s="9" t="n">
-        <x:v>81</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
         <x:v>Rows with parsed INR or USD amount</x:v>
@@ -8438,7 +11162,7 @@
         <x:v>Industry-capability pairs</x:v>
       </x:c>
       <x:c r="B6" s="9" t="n">
-        <x:v>40</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Distinct paired taxonomy combinations</x:v>
@@ -8450,7 +11174,7 @@
         <x:v>Total INR crore</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:v>549476.41</x:v>
+        <x:v>574784.31</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
         <x:v>Parsed chartable INR rows</x:v>
@@ -8478,7 +11202,7 @@
         <x:v>Latest added IDs</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>ai-108, ai-109, ai-110, ai-111, ai-112, ai-113, ai-114, ai-115, ai-116</x:v>
+        <x:v>ai-165, ai-166, ai-167, ai-168, ai-169, ai-170, ai-171, ai-172, ai-173</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
         <x:v>9 newest records</x:v>

</xml_diff>